<commit_message>
MIA: run automatico 2026-08-07 01:10 UTC
</commit_message>
<xml_diff>
--- a/database/AURE3.xlsx
+++ b/database/AURE3.xlsx
@@ -492,16 +492,16 @@
         <v>44650</v>
       </c>
       <c r="B4" t="n">
-        <v>12.38384914398193</v>
+        <v>12.38385009765625</v>
       </c>
       <c r="C4" t="n">
-        <v>13.04504741320321</v>
+        <v>13.04504841779609</v>
       </c>
       <c r="D4" t="n">
-        <v>12.3060608504815</v>
+        <v>12.30606179816537</v>
       </c>
       <c r="E4" t="n">
-        <v>12.9283657147967</v>
+        <v>12.92836671040398</v>
       </c>
       <c r="F4" t="n">
         <v>4408600</v>
@@ -512,16 +512,16 @@
         <v>44651</v>
       </c>
       <c r="B5" t="n">
-        <v>12.4383020401001</v>
+        <v>12.43830108642578</v>
       </c>
       <c r="C5" t="n">
-        <v>12.82724207193696</v>
+        <v>12.82724108844168</v>
       </c>
       <c r="D5" t="n">
-        <v>12.05714098694259</v>
+        <v>12.05714006249281</v>
       </c>
       <c r="E5" t="n">
-        <v>12.41496584590627</v>
+        <v>12.4149648940212</v>
       </c>
       <c r="F5" t="n">
         <v>3876100</v>
@@ -552,16 +552,16 @@
         <v>44655</v>
       </c>
       <c r="B7" t="n">
-        <v>12.42274570465088</v>
+        <v>12.42274475097656</v>
       </c>
       <c r="C7" t="n">
-        <v>12.7338981972699</v>
+        <v>12.7338972197089</v>
       </c>
       <c r="D7" t="n">
-        <v>12.33717841680461</v>
+        <v>12.33717746969916</v>
       </c>
       <c r="E7" t="n">
-        <v>12.54720566311648</v>
+        <v>12.54720469988757</v>
       </c>
       <c r="F7" t="n">
         <v>2842400</v>
@@ -572,16 +572,16 @@
         <v>44656</v>
       </c>
       <c r="B8" t="n">
-        <v>12.15826511383057</v>
+        <v>12.15826606750488</v>
       </c>
       <c r="C8" t="n">
-        <v>12.50053200500811</v>
+        <v>12.50053298552928</v>
       </c>
       <c r="D8" t="n">
-        <v>12.05714061961251</v>
+        <v>12.05714156535479</v>
       </c>
       <c r="E8" t="n">
-        <v>12.37607131730719</v>
+        <v>12.37607228806586</v>
       </c>
       <c r="F8" t="n">
         <v>3624900</v>
@@ -632,16 +632,16 @@
         <v>44659</v>
       </c>
       <c r="B11" t="n">
-        <v>12.60943508148193</v>
+        <v>12.60943603515625</v>
       </c>
       <c r="C11" t="n">
-        <v>12.75723270856147</v>
+        <v>12.75723367341398</v>
       </c>
       <c r="D11" t="n">
-        <v>12.33717750513392</v>
+        <v>12.3371784382169</v>
       </c>
       <c r="E11" t="n">
-        <v>12.33717750513392</v>
+        <v>12.3371784382169</v>
       </c>
       <c r="F11" t="n">
         <v>2049800</v>
@@ -692,16 +692,16 @@
         <v>44664</v>
       </c>
       <c r="B14" t="n">
-        <v>12.10381412506104</v>
+        <v>12.10381317138672</v>
       </c>
       <c r="C14" t="n">
-        <v>12.55498376109398</v>
+        <v>12.55498277187146</v>
       </c>
       <c r="D14" t="n">
-        <v>12.08825616769219</v>
+        <v>12.0882552152437</v>
       </c>
       <c r="E14" t="n">
-        <v>12.39162965978653</v>
+        <v>12.39162868343488</v>
       </c>
       <c r="F14" t="n">
         <v>4421300</v>
@@ -712,16 +712,16 @@
         <v>44665</v>
       </c>
       <c r="B15" t="n">
-        <v>12.11159229278564</v>
+        <v>12.11159324645996</v>
       </c>
       <c r="C15" t="n">
-        <v>12.36829265315281</v>
+        <v>12.36829362703988</v>
       </c>
       <c r="D15" t="n">
-        <v>12.04936194735386</v>
+        <v>12.04936289612812</v>
       </c>
       <c r="E15" t="n">
-        <v>12.08047712006975</v>
+        <v>12.08047807129404</v>
       </c>
       <c r="F15" t="n">
         <v>2077400</v>
@@ -732,16 +732,16 @@
         <v>44669</v>
       </c>
       <c r="B16" t="n">
-        <v>12.45386028289795</v>
+        <v>12.45385932922363</v>
       </c>
       <c r="C16" t="n">
-        <v>12.45386028289795</v>
+        <v>12.45385932922363</v>
       </c>
       <c r="D16" t="n">
-        <v>11.92490159008608</v>
+        <v>11.92490067691762</v>
       </c>
       <c r="E16" t="n">
-        <v>12.10381439459067</v>
+        <v>12.10381346772168</v>
       </c>
       <c r="F16" t="n">
         <v>3931100</v>
@@ -752,16 +752,16 @@
         <v>44670</v>
       </c>
       <c r="B17" t="n">
-        <v>12.10381412506104</v>
+        <v>12.10381317138672</v>
       </c>
       <c r="C17" t="n">
-        <v>12.60165763320052</v>
+        <v>12.60165664030051</v>
       </c>
       <c r="D17" t="n">
-        <v>12.00268962769625</v>
+        <v>12.00268868198966</v>
       </c>
       <c r="E17" t="n">
-        <v>12.4383020482046</v>
+        <v>12.43830106817557</v>
       </c>
       <c r="F17" t="n">
         <v>3118100</v>
@@ -772,16 +772,16 @@
         <v>44671</v>
       </c>
       <c r="B18" t="n">
-        <v>12.05714130401611</v>
+        <v>12.0571403503418</v>
       </c>
       <c r="C18" t="n">
-        <v>12.21271717247328</v>
+        <v>12.2127162064935</v>
       </c>
       <c r="D18" t="n">
-        <v>11.95601680405789</v>
+        <v>11.95601585838214</v>
       </c>
       <c r="E18" t="n">
-        <v>12.07269926178396</v>
+        <v>12.07269830687907</v>
       </c>
       <c r="F18" t="n">
         <v>2798400</v>
@@ -832,16 +832,16 @@
         <v>44677</v>
       </c>
       <c r="B21" t="n">
-        <v>11.95601558685303</v>
+        <v>11.95601654052734</v>
       </c>
       <c r="C21" t="n">
-        <v>12.43830110089237</v>
+        <v>12.4383020930363</v>
       </c>
       <c r="D21" t="n">
-        <v>11.86267007528195</v>
+        <v>11.86267102151054</v>
       </c>
       <c r="E21" t="n">
-        <v>12.32939837498153</v>
+        <v>12.32939935843881</v>
       </c>
       <c r="F21" t="n">
         <v>2627000</v>
@@ -852,16 +852,16 @@
         <v>44678</v>
       </c>
       <c r="B22" t="n">
-        <v>12.05714130401611</v>
+        <v>12.0571403503418</v>
       </c>
       <c r="C22" t="n">
-        <v>12.06492028290003</v>
+        <v>12.06491932861043</v>
       </c>
       <c r="D22" t="n">
-        <v>11.83155610929216</v>
+        <v>11.83155517346078</v>
       </c>
       <c r="E22" t="n">
-        <v>12.04936232513219</v>
+        <v>12.04936137207316</v>
       </c>
       <c r="F22" t="n">
         <v>2401400</v>
@@ -872,16 +872,16 @@
         <v>44679</v>
       </c>
       <c r="B23" t="n">
-        <v>11.90934371948242</v>
+        <v>11.90934467315674</v>
       </c>
       <c r="C23" t="n">
-        <v>12.08825577230682</v>
+        <v>12.08825674030803</v>
       </c>
       <c r="D23" t="n">
-        <v>11.49706676482372</v>
+        <v>11.49706768548379</v>
       </c>
       <c r="E23" t="n">
-        <v>12.08825577230682</v>
+        <v>12.08825674030803</v>
       </c>
       <c r="F23" t="n">
         <v>3489600</v>
@@ -932,16 +932,16 @@
         <v>44684</v>
       </c>
       <c r="B26" t="n">
-        <v>11.27148151397705</v>
+        <v>11.27148246765137</v>
       </c>
       <c r="C26" t="n">
-        <v>11.35704879249248</v>
+        <v>11.3570497534066</v>
       </c>
       <c r="D26" t="n">
-        <v>11.01478116211917</v>
+        <v>11.0147820940742</v>
       </c>
       <c r="E26" t="n">
-        <v>11.15479980562136</v>
+        <v>11.1548007494233</v>
       </c>
       <c r="F26" t="n">
         <v>1672900</v>
@@ -952,16 +952,16 @@
         <v>44685</v>
       </c>
       <c r="B27" t="n">
-        <v>11.69445610046387</v>
+        <v>11.69445705413818</v>
       </c>
       <c r="C27" t="n">
-        <v>11.69445610046387</v>
+        <v>11.69445705413818</v>
       </c>
       <c r="D27" t="n">
-        <v>11.03649597266557</v>
+        <v>11.03649687268372</v>
       </c>
       <c r="E27" t="n">
-        <v>11.20881904113643</v>
+        <v>11.2088199552074</v>
       </c>
       <c r="F27" t="n">
         <v>4400300</v>
@@ -972,16 +972,16 @@
         <v>44686</v>
       </c>
       <c r="B28" t="n">
-        <v>11.28714752197266</v>
+        <v>11.28714847564697</v>
       </c>
       <c r="C28" t="n">
-        <v>11.62396063303483</v>
+        <v>11.62396161516718</v>
       </c>
       <c r="D28" t="n">
-        <v>11.14615584813277</v>
+        <v>11.14615678989441</v>
       </c>
       <c r="E28" t="n">
-        <v>11.61612759626606</v>
+        <v>11.61612857773658</v>
       </c>
       <c r="F28" t="n">
         <v>3065700</v>
@@ -1092,16 +1092,16 @@
         <v>44694</v>
       </c>
       <c r="B34" t="n">
-        <v>11.32631301879883</v>
+        <v>11.32631206512451</v>
       </c>
       <c r="C34" t="n">
-        <v>11.38114278731251</v>
+        <v>11.38114182902154</v>
       </c>
       <c r="D34" t="n">
-        <v>11.11482548824677</v>
+        <v>11.11482455237968</v>
       </c>
       <c r="E34" t="n">
-        <v>11.18532133176413</v>
+        <v>11.18532038996129</v>
       </c>
       <c r="F34" t="n">
         <v>1333500</v>
@@ -1132,16 +1132,16 @@
         <v>44698</v>
       </c>
       <c r="B36" t="n">
-        <v>11.56129837036133</v>
+        <v>11.56129741668701</v>
       </c>
       <c r="C36" t="n">
-        <v>11.74928677955431</v>
+        <v>11.74928581037311</v>
       </c>
       <c r="D36" t="n">
-        <v>11.3576438869025</v>
+        <v>11.35764295002734</v>
       </c>
       <c r="E36" t="n">
-        <v>11.3576438869025</v>
+        <v>11.35764295002734</v>
       </c>
       <c r="F36" t="n">
         <v>1389700</v>
@@ -1152,16 +1152,16 @@
         <v>44699</v>
       </c>
       <c r="B37" t="n">
-        <v>11.1069917678833</v>
+        <v>11.10699272155762</v>
       </c>
       <c r="C37" t="n">
-        <v>11.59262882548476</v>
+        <v>11.5926298208571</v>
       </c>
       <c r="D37" t="n">
-        <v>11.03649593344125</v>
+        <v>11.03649688106261</v>
       </c>
       <c r="E37" t="n">
-        <v>11.51429995454926</v>
+        <v>11.51430094319608</v>
       </c>
       <c r="F37" t="n">
         <v>1959900</v>
@@ -1172,16 +1172,16 @@
         <v>44700</v>
       </c>
       <c r="B38" t="n">
-        <v>11.22448539733887</v>
+        <v>11.22448444366455</v>
       </c>
       <c r="C38" t="n">
-        <v>11.25581679930005</v>
+        <v>11.25581584296371</v>
       </c>
       <c r="D38" t="n">
-        <v>10.97383418164937</v>
+        <v>10.97383324927132</v>
       </c>
       <c r="E38" t="n">
-        <v>11.11482511697494</v>
+        <v>11.11482417261777</v>
       </c>
       <c r="F38" t="n">
         <v>2127500</v>
@@ -1192,16 +1192,16 @@
         <v>44701</v>
       </c>
       <c r="B39" t="n">
-        <v>11.1069917678833</v>
+        <v>11.10699272155762</v>
       </c>
       <c r="C39" t="n">
-        <v>11.34197688669085</v>
+        <v>11.34197786054158</v>
       </c>
       <c r="D39" t="n">
-        <v>10.86417286558284</v>
+        <v>10.86417379840811</v>
       </c>
       <c r="E39" t="n">
-        <v>11.34197688669085</v>
+        <v>11.34197786054158</v>
       </c>
       <c r="F39" t="n">
         <v>1777400</v>
@@ -1232,16 +1232,16 @@
         <v>44705</v>
       </c>
       <c r="B41" t="n">
-        <v>11.21665191650391</v>
+        <v>11.21665096282959</v>
       </c>
       <c r="C41" t="n">
-        <v>11.22448495343431</v>
+        <v>11.22448399909401</v>
       </c>
       <c r="D41" t="n">
-        <v>11.00516514837963</v>
+        <v>11.00516421268657</v>
       </c>
       <c r="E41" t="n">
-        <v>11.09132631361552</v>
+        <v>11.09132537059677</v>
       </c>
       <c r="F41" t="n">
         <v>792900</v>
@@ -1252,16 +1252,16 @@
         <v>44706</v>
       </c>
       <c r="B42" t="n">
-        <v>11.32631301879883</v>
+        <v>11.32631206512451</v>
       </c>
       <c r="C42" t="n">
-        <v>11.39680886231618</v>
+        <v>11.39680790270612</v>
       </c>
       <c r="D42" t="n">
-        <v>11.13832460075227</v>
+        <v>11.13832366290656</v>
       </c>
       <c r="E42" t="n">
-        <v>11.17748904126186</v>
+        <v>11.17748810011851</v>
       </c>
       <c r="F42" t="n">
         <v>821700</v>
@@ -1272,16 +1272,16 @@
         <v>44707</v>
       </c>
       <c r="B43" t="n">
-        <v>11.25581645965576</v>
+        <v>11.25581741333008</v>
       </c>
       <c r="C43" t="n">
-        <v>11.44380486575034</v>
+        <v>11.44380583535239</v>
       </c>
       <c r="D43" t="n">
-        <v>11.20881973163188</v>
+        <v>11.20882068132429</v>
       </c>
       <c r="E43" t="n">
-        <v>11.33414533569493</v>
+        <v>11.33414629600583</v>
       </c>
       <c r="F43" t="n">
         <v>1248800</v>
@@ -1352,16 +1352,16 @@
         <v>44713</v>
       </c>
       <c r="B47" t="n">
-        <v>10.7310152053833</v>
+        <v>10.73101425170898</v>
       </c>
       <c r="C47" t="n">
-        <v>10.94250272786947</v>
+        <v>10.94250175540008</v>
       </c>
       <c r="D47" t="n">
-        <v>10.66051936455458</v>
+        <v>10.66051841714529</v>
       </c>
       <c r="E47" t="n">
-        <v>10.94250272786947</v>
+        <v>10.94250175540008</v>
       </c>
       <c r="F47" t="n">
         <v>6323900</v>
@@ -1372,16 +1372,16 @@
         <v>44714</v>
       </c>
       <c r="B48" t="n">
-        <v>10.86417293548584</v>
+        <v>10.86417388916016</v>
       </c>
       <c r="C48" t="n">
-        <v>10.98949853218943</v>
+        <v>10.98949949686503</v>
       </c>
       <c r="D48" t="n">
-        <v>10.68401757697429</v>
+        <v>10.68401851483428</v>
       </c>
       <c r="E48" t="n">
-        <v>10.75451266487045</v>
+        <v>10.75451360891862</v>
       </c>
       <c r="F48" t="n">
         <v>3275400</v>
@@ -1392,16 +1392,16 @@
         <v>44715</v>
       </c>
       <c r="B49" t="n">
-        <v>10.7780122756958</v>
+        <v>10.77801132202148</v>
       </c>
       <c r="C49" t="n">
-        <v>10.85634040377818</v>
+        <v>10.85633944317314</v>
       </c>
       <c r="D49" t="n">
-        <v>10.62135527253152</v>
+        <v>10.62135433271873</v>
       </c>
       <c r="E49" t="n">
-        <v>10.78584531260389</v>
+        <v>10.78584435823648</v>
       </c>
       <c r="F49" t="n">
         <v>2685000</v>
@@ -1432,16 +1432,16 @@
         <v>44719</v>
       </c>
       <c r="B51" t="n">
-        <v>10.8563404083252</v>
+        <v>10.85634136199951</v>
       </c>
       <c r="C51" t="n">
-        <v>10.87983951905932</v>
+        <v>10.87984047479791</v>
       </c>
       <c r="D51" t="n">
-        <v>10.53519336495403</v>
+        <v>10.53519429041721</v>
       </c>
       <c r="E51" t="n">
-        <v>10.59002387633413</v>
+        <v>10.59002480661389</v>
       </c>
       <c r="F51" t="n">
         <v>2760900</v>
@@ -1532,16 +1532,16 @@
         <v>44726</v>
       </c>
       <c r="B56" t="n">
-        <v>10.39420318603516</v>
+        <v>10.39420223236084</v>
       </c>
       <c r="C56" t="n">
-        <v>10.47253131980584</v>
+        <v>10.47253035894487</v>
       </c>
       <c r="D56" t="n">
-        <v>10.01822560413734</v>
+        <v>10.01822468495919</v>
       </c>
       <c r="E56" t="n">
-        <v>10.01822560413734</v>
+        <v>10.01822468495919</v>
       </c>
       <c r="F56" t="n">
         <v>4085600</v>
@@ -1792,16 +1792,16 @@
         <v>44746</v>
       </c>
       <c r="B69" t="n">
-        <v>10.65268707275391</v>
+        <v>10.65268611907959</v>
       </c>
       <c r="C69" t="n">
-        <v>10.7858457171883</v>
+        <v>10.78584475159305</v>
       </c>
       <c r="D69" t="n">
-        <v>10.52736071852189</v>
+        <v>10.52735977606733</v>
       </c>
       <c r="E69" t="n">
-        <v>10.68401847456203</v>
+        <v>10.68401751808279</v>
       </c>
       <c r="F69" t="n">
         <v>1437100</v>
@@ -1892,16 +1892,16 @@
         <v>44753</v>
       </c>
       <c r="B74" t="n">
-        <v>11.1069917678833</v>
+        <v>11.10699272155762</v>
       </c>
       <c r="C74" t="n">
-        <v>11.18531989181933</v>
+        <v>11.18532085221909</v>
       </c>
       <c r="D74" t="n">
-        <v>10.83284146660853</v>
+        <v>10.83284239674361</v>
       </c>
       <c r="E74" t="n">
-        <v>11.05999429592211</v>
+        <v>11.0599952455611</v>
       </c>
       <c r="F74" t="n">
         <v>1881000</v>
@@ -1912,16 +1912,16 @@
         <v>44754</v>
       </c>
       <c r="B75" t="n">
-        <v>11.14615631103516</v>
+        <v>11.14615535736084</v>
       </c>
       <c r="C75" t="n">
-        <v>11.22448518797689</v>
+        <v>11.22448422760069</v>
       </c>
       <c r="D75" t="n">
-        <v>10.99733234124531</v>
+        <v>10.99733140030449</v>
       </c>
       <c r="E75" t="n">
-        <v>11.10699261956382</v>
+        <v>11.10699166924038</v>
       </c>
       <c r="F75" t="n">
         <v>1673000</v>
@@ -1952,16 +1952,16 @@
         <v>44756</v>
       </c>
       <c r="B77" t="n">
-        <v>10.91117000579834</v>
+        <v>10.91117095947266</v>
       </c>
       <c r="C77" t="n">
-        <v>11.1774872624825</v>
+        <v>11.17748823943387</v>
       </c>
       <c r="D77" t="n">
-        <v>10.84850720975495</v>
+        <v>10.84850815795232</v>
       </c>
       <c r="E77" t="n">
-        <v>11.04432863414042</v>
+        <v>11.04432959945326</v>
       </c>
       <c r="F77" t="n">
         <v>1968500</v>
@@ -1972,16 +1972,16 @@
         <v>44757</v>
       </c>
       <c r="B78" t="n">
-        <v>10.80934429168701</v>
+        <v>10.8093433380127</v>
       </c>
       <c r="C78" t="n">
-        <v>10.98166737847755</v>
+        <v>10.98166640959971</v>
       </c>
       <c r="D78" t="n">
-        <v>10.60568980247997</v>
+        <v>10.60568886677345</v>
       </c>
       <c r="E78" t="n">
-        <v>10.97383434112354</v>
+        <v>10.97383337293678</v>
       </c>
       <c r="F78" t="n">
         <v>2342600</v>
@@ -1992,16 +1992,16 @@
         <v>44760</v>
       </c>
       <c r="B79" t="n">
-        <v>10.7310152053833</v>
+        <v>10.73101425170898</v>
       </c>
       <c r="C79" t="n">
-        <v>11.0051655314951</v>
+        <v>11.00516455345681</v>
       </c>
       <c r="D79" t="n">
-        <v>10.5900242707254</v>
+        <v>10.59002332958107</v>
       </c>
       <c r="E79" t="n">
-        <v>10.80934408341511</v>
+        <v>10.80934312277964</v>
       </c>
       <c r="F79" t="n">
         <v>1463400</v>
@@ -2012,16 +2012,16 @@
         <v>44761</v>
       </c>
       <c r="B80" t="n">
-        <v>11.0913257598877</v>
+        <v>11.09132671356201</v>
       </c>
       <c r="C80" t="n">
-        <v>11.0913257598877</v>
+        <v>11.09132671356201</v>
       </c>
       <c r="D80" t="n">
-        <v>10.78584480484809</v>
+        <v>10.78584573225599</v>
       </c>
       <c r="E80" t="n">
-        <v>10.87200596578243</v>
+        <v>10.87200690059879</v>
       </c>
       <c r="F80" t="n">
         <v>2890800</v>
@@ -2132,16 +2132,16 @@
         <v>44769</v>
       </c>
       <c r="B86" t="n">
-        <v>11.24015140533447</v>
+        <v>11.24015045166016</v>
       </c>
       <c r="C86" t="n">
-        <v>11.49080261954139</v>
+        <v>11.49080164460048</v>
       </c>
       <c r="D86" t="n">
-        <v>11.15398949020119</v>
+        <v>11.15398854383731</v>
       </c>
       <c r="E86" t="n">
-        <v>11.2871481344985</v>
+        <v>11.28714717683673</v>
       </c>
       <c r="F86" t="n">
         <v>3096400</v>
@@ -2152,16 +2152,16 @@
         <v>44770</v>
       </c>
       <c r="B87" t="n">
-        <v>10.9660005569458</v>
+        <v>10.96600151062012</v>
       </c>
       <c r="C87" t="n">
-        <v>11.33414507051741</v>
+        <v>11.33414605620796</v>
       </c>
       <c r="D87" t="n">
-        <v>10.8250088821738</v>
+        <v>10.82500982358657</v>
       </c>
       <c r="E87" t="n">
-        <v>11.31064596005574</v>
+        <v>11.31064694370265</v>
       </c>
       <c r="F87" t="n">
         <v>2911900</v>
@@ -2212,16 +2212,16 @@
         <v>44775</v>
       </c>
       <c r="B90" t="n">
-        <v>10.86417293548584</v>
+        <v>10.86417388916016</v>
       </c>
       <c r="C90" t="n">
-        <v>11.06782740362892</v>
+        <v>11.06782837518035</v>
       </c>
       <c r="D90" t="n">
-        <v>10.72318126569455</v>
+        <v>10.7231822069924</v>
       </c>
       <c r="E90" t="n">
-        <v>10.93466877038148</v>
+        <v>10.93466973024404</v>
       </c>
       <c r="F90" t="n">
         <v>2371400</v>
@@ -2232,16 +2232,16 @@
         <v>44776</v>
       </c>
       <c r="B91" t="n">
-        <v>10.88767147064209</v>
+        <v>10.88767242431641</v>
       </c>
       <c r="C91" t="n">
-        <v>11.02083010599954</v>
+        <v>11.02083107133751</v>
       </c>
       <c r="D91" t="n">
-        <v>10.70751610927583</v>
+        <v>10.70751704716995</v>
       </c>
       <c r="E91" t="n">
-        <v>10.83284170796531</v>
+        <v>10.83284265683698</v>
       </c>
       <c r="F91" t="n">
         <v>3133200</v>
@@ -2272,16 +2272,16 @@
         <v>44778</v>
       </c>
       <c r="B93" t="n">
-        <v>10.9660005569458</v>
+        <v>10.96600151062012</v>
       </c>
       <c r="C93" t="n">
-        <v>11.16965503228325</v>
+        <v>11.16965600366867</v>
       </c>
       <c r="D93" t="n">
-        <v>10.93466915666308</v>
+        <v>10.93467010761261</v>
       </c>
       <c r="E93" t="n">
-        <v>11.16965503228325</v>
+        <v>11.16965600366867</v>
       </c>
       <c r="F93" t="n">
         <v>1948700</v>
@@ -2312,16 +2312,16 @@
         <v>44782</v>
       </c>
       <c r="B95" t="n">
-        <v>10.92683696746826</v>
+        <v>10.92683601379395</v>
       </c>
       <c r="C95" t="n">
-        <v>11.0599956157492</v>
+        <v>11.05999465045304</v>
       </c>
       <c r="D95" t="n">
-        <v>10.67618574576276</v>
+        <v>10.67618481396482</v>
       </c>
       <c r="E95" t="n">
-        <v>10.98166748246601</v>
+        <v>10.98166652400619</v>
       </c>
       <c r="F95" t="n">
         <v>1743500</v>
@@ -2392,16 +2392,16 @@
         <v>44788</v>
       </c>
       <c r="B99" t="n">
-        <v>11.21665191650391</v>
+        <v>11.21665096282959</v>
       </c>
       <c r="C99" t="n">
-        <v>11.3106461186702</v>
+        <v>11.3106451570042</v>
       </c>
       <c r="D99" t="n">
-        <v>10.92683627307463</v>
+        <v>10.92683534404133</v>
       </c>
       <c r="E99" t="n">
-        <v>10.99733211144923</v>
+        <v>10.99733117642216</v>
       </c>
       <c r="F99" t="n">
         <v>3450900</v>
@@ -2432,16 +2432,16 @@
         <v>44790</v>
       </c>
       <c r="B101" t="n">
-        <v>11.24015140533447</v>
+        <v>11.24015045166016</v>
       </c>
       <c r="C101" t="n">
-        <v>11.25581673272263</v>
+        <v>11.25581577771919</v>
       </c>
       <c r="D101" t="n">
-        <v>10.91117131318813</v>
+        <v>10.91117038742624</v>
       </c>
       <c r="E101" t="n">
-        <v>10.98949944412802</v>
+        <v>10.98949851172035</v>
       </c>
       <c r="F101" t="n">
         <v>4396400</v>
@@ -2492,16 +2492,16 @@
         <v>44795</v>
       </c>
       <c r="B104" t="n">
-        <v>11.0599946975708</v>
+        <v>11.05999565124512</v>
       </c>
       <c r="C104" t="n">
-        <v>11.2244847349093</v>
+        <v>11.22448570276716</v>
       </c>
       <c r="D104" t="n">
-        <v>10.98166657079026</v>
+        <v>10.98166751771054</v>
       </c>
       <c r="E104" t="n">
-        <v>11.0599946975708</v>
+        <v>11.05999565124512</v>
       </c>
       <c r="F104" t="n">
         <v>1703300</v>
@@ -2512,16 +2512,16 @@
         <v>44796</v>
       </c>
       <c r="B105" t="n">
-        <v>11.22448539733887</v>
+        <v>11.22448444366455</v>
       </c>
       <c r="C105" t="n">
-        <v>11.27148287378042</v>
+        <v>11.27148191611302</v>
       </c>
       <c r="D105" t="n">
-        <v>10.98949950913019</v>
+        <v>10.98949857542116</v>
       </c>
       <c r="E105" t="n">
-        <v>10.98949950913019</v>
+        <v>10.98949857542116</v>
       </c>
       <c r="F105" t="n">
         <v>2361000</v>
@@ -2532,16 +2532,16 @@
         <v>44797</v>
       </c>
       <c r="B106" t="n">
-        <v>11.1069917678833</v>
+        <v>11.10699272155762</v>
       </c>
       <c r="C106" t="n">
-        <v>11.39680739514549</v>
+        <v>11.3968083737041</v>
       </c>
       <c r="D106" t="n">
-        <v>11.09915873138986</v>
+        <v>11.09915968439161</v>
       </c>
       <c r="E106" t="n">
-        <v>11.22448432728707</v>
+        <v>11.2244852910496</v>
       </c>
       <c r="F106" t="n">
         <v>2116800</v>
@@ -2632,16 +2632,16 @@
         <v>44804</v>
       </c>
       <c r="B111" t="n">
-        <v>12.03910160064697</v>
+        <v>12.03910255432129</v>
       </c>
       <c r="C111" t="n">
-        <v>12.07826603661254</v>
+        <v>12.07826699338926</v>
       </c>
       <c r="D111" t="n">
-        <v>10.96600023838756</v>
+        <v>10.96600110705643</v>
       </c>
       <c r="E111" t="n">
-        <v>11.02083000053966</v>
+        <v>11.02083087355185</v>
       </c>
       <c r="F111" t="n">
         <v>16560000</v>
@@ -2652,16 +2652,16 @@
         <v>44805</v>
       </c>
       <c r="B112" t="n">
-        <v>11.65529251098633</v>
+        <v>11.65529346466064</v>
       </c>
       <c r="C112" t="n">
-        <v>12.15659567974902</v>
+        <v>12.1565966744416</v>
       </c>
       <c r="D112" t="n">
-        <v>11.42030662728508</v>
+        <v>11.42030756173208</v>
       </c>
       <c r="E112" t="n">
-        <v>12.14092960556915</v>
+        <v>12.14093059897989</v>
       </c>
       <c r="F112" t="n">
         <v>4716400</v>
@@ -2712,16 +2712,16 @@
         <v>44810</v>
       </c>
       <c r="B115" t="n">
-        <v>11.58479785919189</v>
+        <v>11.58479595184326</v>
       </c>
       <c r="C115" t="n">
-        <v>11.90594494281729</v>
+        <v>11.90594298259424</v>
       </c>
       <c r="D115" t="n">
-        <v>11.49863668336545</v>
+        <v>11.49863479020259</v>
       </c>
       <c r="E115" t="n">
-        <v>11.89811190492408</v>
+        <v>11.89810994599068</v>
       </c>
       <c r="F115" t="n">
         <v>1316500</v>
@@ -2792,16 +2792,16 @@
         <v>44817</v>
       </c>
       <c r="B119" t="n">
-        <v>11.24015140533447</v>
+        <v>11.24015045166016</v>
       </c>
       <c r="C119" t="n">
-        <v>11.43597285318351</v>
+        <v>11.43597188289466</v>
       </c>
       <c r="D119" t="n">
-        <v>11.16965556458889</v>
+        <v>11.16965461689582</v>
       </c>
       <c r="E119" t="n">
-        <v>11.3028142088862</v>
+        <v>11.30281324989524</v>
       </c>
       <c r="F119" t="n">
         <v>1768400</v>
@@ -2832,16 +2832,16 @@
         <v>44819</v>
       </c>
       <c r="B121" t="n">
-        <v>11.22448539733887</v>
+        <v>11.22448444366455</v>
       </c>
       <c r="C121" t="n">
-        <v>11.27148287378042</v>
+        <v>11.27148191611302</v>
       </c>
       <c r="D121" t="n">
-        <v>11.11482511697494</v>
+        <v>11.11482417261777</v>
       </c>
       <c r="E121" t="n">
-        <v>11.16182259341649</v>
+        <v>11.16182164506624</v>
       </c>
       <c r="F121" t="n">
         <v>1523500</v>
@@ -2872,16 +2872,16 @@
         <v>44823</v>
       </c>
       <c r="B123" t="n">
-        <v>11.28714752197266</v>
+        <v>11.28714847564697</v>
       </c>
       <c r="C123" t="n">
-        <v>11.43597223258132</v>
+        <v>11.43597319883014</v>
       </c>
       <c r="D123" t="n">
-        <v>11.11482444805718</v>
+        <v>11.11482538717157</v>
       </c>
       <c r="E123" t="n">
-        <v>11.11482444805718</v>
+        <v>11.11482538717157</v>
       </c>
       <c r="F123" t="n">
         <v>1858600</v>
@@ -2892,16 +2892,16 @@
         <v>44824</v>
       </c>
       <c r="B124" t="n">
-        <v>11.13049125671387</v>
+        <v>11.13049030303955</v>
       </c>
       <c r="C124" t="n">
-        <v>11.35764410901417</v>
+        <v>11.35764313587711</v>
       </c>
       <c r="D124" t="n">
-        <v>11.08349377999676</v>
+        <v>11.08349283034925</v>
       </c>
       <c r="E124" t="n">
-        <v>11.28714826743829</v>
+        <v>11.28714730034141</v>
       </c>
       <c r="F124" t="n">
         <v>1310600</v>
@@ -2912,16 +2912,16 @@
         <v>44825</v>
       </c>
       <c r="B125" t="n">
-        <v>11.0913257598877</v>
+        <v>11.09132671356201</v>
       </c>
       <c r="C125" t="n">
-        <v>11.23231742959796</v>
+        <v>11.23231839539528</v>
       </c>
       <c r="D125" t="n">
-        <v>10.93466876409822</v>
+        <v>10.93466970430257</v>
       </c>
       <c r="E125" t="n">
-        <v>11.13049019558493</v>
+        <v>11.13049115262676</v>
       </c>
       <c r="F125" t="n">
         <v>2825100</v>
@@ -2992,16 +2992,16 @@
         <v>44831</v>
       </c>
       <c r="B129" t="n">
-        <v>10.9033374786377</v>
+        <v>10.90333843231201</v>
       </c>
       <c r="C129" t="n">
-        <v>11.04432914981819</v>
+        <v>11.04433011582452</v>
       </c>
       <c r="D129" t="n">
-        <v>10.77017884407822</v>
+        <v>10.77017978610565</v>
       </c>
       <c r="E129" t="n">
-        <v>11.04432914981819</v>
+        <v>11.04433011582452</v>
       </c>
       <c r="F129" t="n">
         <v>2130200</v>
@@ -3032,16 +3032,16 @@
         <v>44833</v>
       </c>
       <c r="B131" t="n">
-        <v>10.70751571655273</v>
+        <v>10.70751667022705</v>
       </c>
       <c r="C131" t="n">
-        <v>10.83284131064561</v>
+        <v>10.83284227548216</v>
       </c>
       <c r="D131" t="n">
-        <v>10.6448529195063</v>
+        <v>10.6448538675995</v>
       </c>
       <c r="E131" t="n">
-        <v>10.69184964379139</v>
+        <v>10.6918505960704</v>
       </c>
       <c r="F131" t="n">
         <v>2222600</v>
@@ -3132,16 +3132,16 @@
         <v>44840</v>
       </c>
       <c r="B136" t="n">
-        <v>10.98950004577637</v>
+        <v>10.98949909210205</v>
       </c>
       <c r="C136" t="n">
-        <v>11.12265869736379</v>
+        <v>11.1226577321339</v>
       </c>
       <c r="D136" t="n">
-        <v>10.88767279768013</v>
+        <v>10.88767185284243</v>
       </c>
       <c r="E136" t="n">
-        <v>11.02866448689024</v>
+        <v>11.02866352981721</v>
       </c>
       <c r="F136" t="n">
         <v>3101100</v>
@@ -3192,16 +3192,16 @@
         <v>44845</v>
       </c>
       <c r="B139" t="n">
-        <v>11.22448539733887</v>
+        <v>11.22448444366455</v>
       </c>
       <c r="C139" t="n">
-        <v>11.31847960322243</v>
+        <v>11.31847864156201</v>
       </c>
       <c r="D139" t="n">
-        <v>10.99733254637037</v>
+        <v>10.99733161199581</v>
       </c>
       <c r="E139" t="n">
-        <v>11.04433002281193</v>
+        <v>11.04432908444429</v>
       </c>
       <c r="F139" t="n">
         <v>1834300</v>
@@ -3212,16 +3212,16 @@
         <v>44847</v>
       </c>
       <c r="B140" t="n">
-        <v>10.91117000579834</v>
+        <v>10.91117095947266</v>
       </c>
       <c r="C140" t="n">
-        <v>11.20098562424891</v>
+        <v>11.20098660325412</v>
       </c>
       <c r="D140" t="n">
-        <v>10.87200557152136</v>
+        <v>10.87200652177256</v>
       </c>
       <c r="E140" t="n">
-        <v>11.12265675569494</v>
+        <v>11.12265772785393</v>
       </c>
       <c r="F140" t="n">
         <v>3739400</v>
@@ -3292,16 +3292,16 @@
         <v>44853</v>
       </c>
       <c r="B144" t="n">
-        <v>11.02083015441895</v>
+        <v>11.02082920074463</v>
       </c>
       <c r="C144" t="n">
-        <v>11.3263118628163</v>
+        <v>11.32631088270749</v>
       </c>
       <c r="D144" t="n">
-        <v>10.9973317913113</v>
+        <v>10.99733083967039</v>
       </c>
       <c r="E144" t="n">
-        <v>11.2871474263039</v>
+        <v>11.28714644958413</v>
       </c>
       <c r="F144" t="n">
         <v>2951600</v>
@@ -3372,16 +3372,16 @@
         <v>44859</v>
       </c>
       <c r="B148" t="n">
-        <v>11.38897609710693</v>
+        <v>11.3889741897583</v>
       </c>
       <c r="C148" t="n">
-        <v>11.5064686744452</v>
+        <v>11.50646674741971</v>
       </c>
       <c r="D148" t="n">
-        <v>11.18532159918765</v>
+        <v>11.18531972594569</v>
       </c>
       <c r="E148" t="n">
-        <v>11.24015211601182</v>
+        <v>11.24015023358722</v>
       </c>
       <c r="F148" t="n">
         <v>2935500</v>
@@ -3392,16 +3392,16 @@
         <v>44860</v>
       </c>
       <c r="B149" t="n">
-        <v>11.34197807312012</v>
+        <v>11.3419771194458</v>
       </c>
       <c r="C149" t="n">
-        <v>11.45163835450095</v>
+        <v>11.451637391606</v>
       </c>
       <c r="D149" t="n">
-        <v>11.20098713648711</v>
+        <v>11.20098619466782</v>
       </c>
       <c r="E149" t="n">
-        <v>11.43597302687486</v>
+        <v>11.43597206529711</v>
       </c>
       <c r="F149" t="n">
         <v>4386900</v>
@@ -3432,16 +3432,16 @@
         <v>44862</v>
       </c>
       <c r="B151" t="n">
-        <v>11.49080181121826</v>
+        <v>11.49080276489258</v>
       </c>
       <c r="C151" t="n">
-        <v>11.63962577243467</v>
+        <v>11.63962673846057</v>
       </c>
       <c r="D151" t="n">
-        <v>11.2244845413578</v>
+        <v>11.22448547292922</v>
       </c>
       <c r="E151" t="n">
-        <v>11.32631177671618</v>
+        <v>11.32631271673871</v>
       </c>
       <c r="F151" t="n">
         <v>2887600</v>
@@ -3452,16 +3452,16 @@
         <v>44865</v>
       </c>
       <c r="B152" t="n">
-        <v>11.68662357330322</v>
+        <v>11.68662452697754</v>
       </c>
       <c r="C152" t="n">
-        <v>11.72578801061714</v>
+        <v>11.72578896748743</v>
       </c>
       <c r="D152" t="n">
-        <v>11.16182205549541</v>
+        <v>11.16182296634386</v>
       </c>
       <c r="E152" t="n">
-        <v>11.23231789326056</v>
+        <v>11.23231880986175</v>
       </c>
       <c r="F152" t="n">
         <v>2644000</v>
@@ -3492,16 +3492,16 @@
         <v>44868</v>
       </c>
       <c r="B154" t="n">
-        <v>11.68662357330322</v>
+        <v>11.68662452697754</v>
       </c>
       <c r="C154" t="n">
-        <v>11.74928637420569</v>
+        <v>11.74928733299354</v>
       </c>
       <c r="D154" t="n">
-        <v>11.36547653192819</v>
+        <v>11.36547745939565</v>
       </c>
       <c r="E154" t="n">
-        <v>11.49863517059581</v>
+        <v>11.49863610892954</v>
       </c>
       <c r="F154" t="n">
         <v>2959500</v>
@@ -3592,16 +3592,16 @@
         <v>44875</v>
       </c>
       <c r="B159" t="n">
-        <v>10.70751571655273</v>
+        <v>10.70751667022705</v>
       </c>
       <c r="C159" t="n">
-        <v>11.10699160797338</v>
+        <v>11.10699259722736</v>
       </c>
       <c r="D159" t="n">
-        <v>10.49602821627141</v>
+        <v>10.4960291511094</v>
       </c>
       <c r="E159" t="n">
-        <v>11.04432881092694</v>
+        <v>11.04432979459981</v>
       </c>
       <c r="F159" t="n">
         <v>4341400</v>
@@ -3612,16 +3612,16 @@
         <v>44876</v>
       </c>
       <c r="B160" t="n">
-        <v>10.79367828369141</v>
+        <v>10.79367733001709</v>
       </c>
       <c r="C160" t="n">
-        <v>10.85634108891171</v>
+        <v>10.85634012970083</v>
       </c>
       <c r="D160" t="n">
-        <v>10.53519402540776</v>
+        <v>10.5351930945718</v>
       </c>
       <c r="E160" t="n">
-        <v>10.78584599328854</v>
+        <v>10.78584504030624</v>
       </c>
       <c r="F160" t="n">
         <v>3291200</v>
@@ -3652,16 +3652,16 @@
         <v>44881</v>
       </c>
       <c r="B162" t="n">
-        <v>10.9033374786377</v>
+        <v>10.90333843231201</v>
       </c>
       <c r="C162" t="n">
-        <v>10.9033374786377</v>
+        <v>10.90333843231201</v>
       </c>
       <c r="D162" t="n">
-        <v>10.59785577341312</v>
+        <v>10.59785670036809</v>
       </c>
       <c r="E162" t="n">
-        <v>10.86417304253206</v>
+        <v>10.86417399278081</v>
       </c>
       <c r="F162" t="n">
         <v>5270300</v>
@@ -3692,16 +3692,16 @@
         <v>44883</v>
       </c>
       <c r="B164" t="n">
-        <v>10.78584671020508</v>
+        <v>10.78584575653076</v>
       </c>
       <c r="C164" t="n">
-        <v>10.9895004672078</v>
+        <v>10.98949949552661</v>
       </c>
       <c r="D164" t="n">
-        <v>10.57435916827967</v>
+        <v>10.57435823330488</v>
       </c>
       <c r="E164" t="n">
-        <v>10.8093450769747</v>
+        <v>10.80934412122268</v>
       </c>
       <c r="F164" t="n">
         <v>3568700</v>
@@ -3732,16 +3732,16 @@
         <v>44887</v>
       </c>
       <c r="B166" t="n">
-        <v>10.84850883483887</v>
+        <v>10.84850788116455</v>
       </c>
       <c r="C166" t="n">
-        <v>11.4203071211389</v>
+        <v>11.42030611719874</v>
       </c>
       <c r="D166" t="n">
-        <v>10.80151135726647</v>
+        <v>10.80151040772362</v>
       </c>
       <c r="E166" t="n">
-        <v>11.29498151027859</v>
+        <v>11.29498051735561</v>
       </c>
       <c r="F166" t="n">
         <v>3523700</v>
@@ -3752,16 +3752,16 @@
         <v>44888</v>
       </c>
       <c r="B167" t="n">
-        <v>10.56652450561523</v>
+        <v>10.56652545928955</v>
       </c>
       <c r="C167" t="n">
-        <v>10.8171764516154</v>
+        <v>10.81717742791213</v>
       </c>
       <c r="D167" t="n">
-        <v>10.51952777930236</v>
+        <v>10.51952872873502</v>
       </c>
       <c r="E167" t="n">
-        <v>10.80934341489675</v>
+        <v>10.80934439048652</v>
       </c>
       <c r="F167" t="n">
         <v>4669400</v>
@@ -3872,16 +3872,16 @@
         <v>44896</v>
       </c>
       <c r="B173" t="n">
-        <v>10.92683696746826</v>
+        <v>10.92683601379395</v>
       </c>
       <c r="C173" t="n">
-        <v>11.02083117560783</v>
+        <v>11.02083021372987</v>
       </c>
       <c r="D173" t="n">
-        <v>10.69185107361957</v>
+        <v>10.69185014045439</v>
       </c>
       <c r="E173" t="n">
-        <v>10.76234691647413</v>
+        <v>10.76234597715621</v>
       </c>
       <c r="F173" t="n">
         <v>1944500</v>
@@ -3892,16 +3892,16 @@
         <v>44897</v>
       </c>
       <c r="B174" t="n">
-        <v>10.80151081085205</v>
+        <v>10.80150985717773</v>
       </c>
       <c r="C174" t="n">
-        <v>11.09132645805553</v>
+        <v>11.09132547879316</v>
       </c>
       <c r="D174" t="n">
-        <v>10.79367777381964</v>
+        <v>10.79367682083691</v>
       </c>
       <c r="E174" t="n">
-        <v>10.92683641537253</v>
+        <v>10.92683545063311</v>
       </c>
       <c r="F174" t="n">
         <v>1109200</v>
@@ -3912,16 +3912,16 @@
         <v>44900</v>
       </c>
       <c r="B175" t="n">
-        <v>10.51952743530273</v>
+        <v>10.51952838897705</v>
       </c>
       <c r="C175" t="n">
-        <v>10.80151002495736</v>
+        <v>10.80151100419552</v>
       </c>
       <c r="D175" t="n">
-        <v>10.50386136237774</v>
+        <v>10.50386231463181</v>
       </c>
       <c r="E175" t="n">
-        <v>10.77801166256934</v>
+        <v>10.7780126396772</v>
       </c>
       <c r="F175" t="n">
         <v>1355000</v>
@@ -3932,16 +3932,16 @@
         <v>44901</v>
       </c>
       <c r="B176" t="n">
-        <v>10.47253036499023</v>
+        <v>10.47253131866455</v>
       </c>
       <c r="C176" t="n">
-        <v>10.58219063867058</v>
+        <v>10.58219160233104</v>
       </c>
       <c r="D176" t="n">
-        <v>10.41770060164981</v>
+        <v>10.41770155033109</v>
       </c>
       <c r="E176" t="n">
-        <v>10.51952783856738</v>
+        <v>10.51952879652149</v>
       </c>
       <c r="F176" t="n">
         <v>1647500</v>
@@ -3952,16 +3952,16 @@
         <v>44902</v>
       </c>
       <c r="B177" t="n">
-        <v>10.65268707275391</v>
+        <v>10.65268611907959</v>
       </c>
       <c r="C177" t="n">
-        <v>10.80151104459258</v>
+        <v>10.80151007759491</v>
       </c>
       <c r="D177" t="n">
-        <v>10.42553422289516</v>
+        <v>10.42553328955654</v>
       </c>
       <c r="E177" t="n">
-        <v>10.42553422289516</v>
+        <v>10.42553328955654</v>
       </c>
       <c r="F177" t="n">
         <v>2865300</v>
@@ -3972,16 +3972,16 @@
         <v>44903</v>
       </c>
       <c r="B178" t="n">
-        <v>11.26364898681641</v>
+        <v>11.26364994049072</v>
       </c>
       <c r="C178" t="n">
-        <v>11.8119488532735</v>
+        <v>11.81194985337145</v>
       </c>
       <c r="D178" t="n">
-        <v>11.15398871472519</v>
+        <v>11.15398965911476</v>
       </c>
       <c r="E178" t="n">
-        <v>11.74928605407837</v>
+        <v>11.74928704887077</v>
       </c>
       <c r="F178" t="n">
         <v>12105700</v>
@@ -4052,16 +4052,16 @@
         <v>44909</v>
       </c>
       <c r="B182" t="n">
-        <v>10.99733257293701</v>
+        <v>10.9973316192627</v>
       </c>
       <c r="C182" t="n">
-        <v>11.13832425560273</v>
+        <v>11.13832328970179</v>
       </c>
       <c r="D182" t="n">
-        <v>10.7388483193829</v>
+        <v>10.738847388124</v>
       </c>
       <c r="E182" t="n">
-        <v>11.01299864745522</v>
+        <v>11.01299769242237</v>
       </c>
       <c r="F182" t="n">
         <v>3892800</v>
@@ -4152,16 +4152,16 @@
         <v>44916</v>
       </c>
       <c r="B187" t="n">
-        <v>11.58479785919189</v>
+        <v>11.58479595184326</v>
       </c>
       <c r="C187" t="n">
-        <v>11.7571209578444</v>
+        <v>11.75711902212409</v>
       </c>
       <c r="D187" t="n">
-        <v>11.15399048606043</v>
+        <v>11.15398864964095</v>
       </c>
       <c r="E187" t="n">
-        <v>11.4281408363258</v>
+        <v>11.42813895476955</v>
       </c>
       <c r="F187" t="n">
         <v>6348400</v>
@@ -4192,16 +4192,16 @@
         <v>44918</v>
       </c>
       <c r="B189" t="n">
-        <v>11.78845119476318</v>
+        <v>11.78845024108887</v>
       </c>
       <c r="C189" t="n">
-        <v>12.09393217234406</v>
+        <v>12.09393119395663</v>
       </c>
       <c r="D189" t="n">
-        <v>11.57696367459224</v>
+        <v>11.57696273802706</v>
       </c>
       <c r="E189" t="n">
-        <v>11.67879091611904</v>
+        <v>11.67878997131614</v>
       </c>
       <c r="F189" t="n">
         <v>5656000</v>
@@ -4232,16 +4232,16 @@
         <v>44922</v>
       </c>
       <c r="B191" t="n">
-        <v>11.52996730804443</v>
+        <v>11.52996635437012</v>
       </c>
       <c r="C191" t="n">
-        <v>11.60829544067951</v>
+        <v>11.60829448052647</v>
       </c>
       <c r="D191" t="n">
-        <v>11.34197814632122</v>
+        <v>11.34197720819598</v>
       </c>
       <c r="E191" t="n">
-        <v>11.60829544067951</v>
+        <v>11.60829448052647</v>
       </c>
       <c r="F191" t="n">
         <v>1633000</v>
@@ -4252,16 +4252,16 @@
         <v>44923</v>
       </c>
       <c r="B192" t="n">
-        <v>11.58479785919189</v>
+        <v>11.58479595184326</v>
       </c>
       <c r="C192" t="n">
-        <v>11.69445814869797</v>
+        <v>11.6944562232946</v>
       </c>
       <c r="D192" t="n">
-        <v>11.49863668336545</v>
+        <v>11.49863479020259</v>
       </c>
       <c r="E192" t="n">
-        <v>11.57696482129869</v>
+        <v>11.5769629152397</v>
       </c>
       <c r="F192" t="n">
         <v>2005900</v>
@@ -4272,16 +4272,16 @@
         <v>44924</v>
       </c>
       <c r="B193" t="n">
-        <v>11.53779983520508</v>
+        <v>11.53779888153076</v>
       </c>
       <c r="C193" t="n">
-        <v>11.73362129131107</v>
+        <v>11.73362032145083</v>
       </c>
       <c r="D193" t="n">
-        <v>11.47513702901113</v>
+        <v>11.4751360805163</v>
       </c>
       <c r="E193" t="n">
-        <v>11.62396175397144</v>
+        <v>11.62396079317528</v>
       </c>
       <c r="F193" t="n">
         <v>2424800</v>
@@ -4292,16 +4292,16 @@
         <v>44928</v>
       </c>
       <c r="B194" t="n">
-        <v>11.34197807312012</v>
+        <v>11.3419771194458</v>
       </c>
       <c r="C194" t="n">
-        <v>11.46730442912659</v>
+        <v>11.46730346491438</v>
       </c>
       <c r="D194" t="n">
-        <v>11.1774887715482</v>
+        <v>11.17748783170473</v>
       </c>
       <c r="E194" t="n">
-        <v>11.38897554999749</v>
+        <v>11.38897459237146</v>
       </c>
       <c r="F194" t="n">
         <v>1018800</v>
@@ -4372,16 +4372,16 @@
         <v>44932</v>
       </c>
       <c r="B198" t="n">
-        <v>11.42030620574951</v>
+        <v>11.4203052520752</v>
       </c>
       <c r="C198" t="n">
-        <v>11.53779876976359</v>
+        <v>11.53779780627784</v>
       </c>
       <c r="D198" t="n">
-        <v>11.31847896833754</v>
+        <v>11.3184780231665</v>
       </c>
       <c r="E198" t="n">
-        <v>11.4124731689487</v>
+        <v>11.4124722159285</v>
       </c>
       <c r="F198" t="n">
         <v>2864500</v>
@@ -4472,16 +4472,16 @@
         <v>44939</v>
       </c>
       <c r="B203" t="n">
-        <v>11.58479785919189</v>
+        <v>11.58479595184326</v>
       </c>
       <c r="C203" t="n">
-        <v>11.78845236241762</v>
+        <v>11.78845042153883</v>
       </c>
       <c r="D203" t="n">
-        <v>11.4438061651126</v>
+        <v>11.44380428097718</v>
       </c>
       <c r="E203" t="n">
-        <v>11.7492879199512</v>
+        <v>11.74928598552053</v>
       </c>
       <c r="F203" t="n">
         <v>2269100</v>
@@ -4492,16 +4492,16 @@
         <v>44942</v>
       </c>
       <c r="B204" t="n">
-        <v>11.78845119476318</v>
+        <v>11.78845024108887</v>
       </c>
       <c r="C204" t="n">
-        <v>11.80411652199833</v>
+        <v>11.8041155670567</v>
       </c>
       <c r="D204" t="n">
-        <v>11.39680830289065</v>
+        <v>11.39680738089987</v>
       </c>
       <c r="E204" t="n">
-        <v>11.49080250730011</v>
+        <v>11.49080157770529</v>
       </c>
       <c r="F204" t="n">
         <v>3279700</v>
@@ -4512,16 +4512,16 @@
         <v>44943</v>
       </c>
       <c r="B205" t="n">
-        <v>11.74928569793701</v>
+        <v>11.74928665161133</v>
       </c>
       <c r="C205" t="n">
-        <v>11.93727408982413</v>
+        <v>11.93727505875722</v>
       </c>
       <c r="D205" t="n">
-        <v>11.60829403052194</v>
+        <v>11.60829497275214</v>
       </c>
       <c r="E205" t="n">
-        <v>11.81194849523272</v>
+        <v>11.81194945399329</v>
       </c>
       <c r="F205" t="n">
         <v>2676600</v>
@@ -4572,16 +4572,16 @@
         <v>44946</v>
       </c>
       <c r="B208" t="n">
-        <v>11.58479785919189</v>
+        <v>11.58479595184326</v>
       </c>
       <c r="C208" t="n">
-        <v>11.68662511080476</v>
+        <v>11.68662318669104</v>
       </c>
       <c r="D208" t="n">
-        <v>11.48297060757903</v>
+        <v>11.48296871699548</v>
       </c>
       <c r="E208" t="n">
-        <v>11.65529370623154</v>
+        <v>11.6552917872763</v>
       </c>
       <c r="F208" t="n">
         <v>2012100</v>
@@ -4612,16 +4612,16 @@
         <v>44950</v>
       </c>
       <c r="B210" t="n">
-        <v>11.68662357330322</v>
+        <v>11.68662452697754</v>
       </c>
       <c r="C210" t="n">
-        <v>11.80411613824548</v>
+        <v>11.80411710150764</v>
       </c>
       <c r="D210" t="n">
-        <v>11.32631209461427</v>
+        <v>11.32631301888575</v>
       </c>
       <c r="E210" t="n">
-        <v>11.52996657104705</v>
+        <v>11.52996751193754</v>
       </c>
       <c r="F210" t="n">
         <v>5839900</v>
@@ -4632,16 +4632,16 @@
         <v>44951</v>
       </c>
       <c r="B211" t="n">
-        <v>11.89027786254883</v>
+        <v>11.89027881622314</v>
       </c>
       <c r="C211" t="n">
-        <v>12.07043322555739</v>
+        <v>12.07043419368129</v>
       </c>
       <c r="D211" t="n">
-        <v>11.62396058940618</v>
+        <v>11.62396152172019</v>
       </c>
       <c r="E211" t="n">
-        <v>11.67879035258278</v>
+        <v>11.67879128929448</v>
       </c>
       <c r="F211" t="n">
         <v>10764800</v>
@@ -4712,16 +4712,16 @@
         <v>44957</v>
       </c>
       <c r="B215" t="n">
-        <v>12.07043361663818</v>
+        <v>12.0704345703125</v>
       </c>
       <c r="C215" t="n">
-        <v>12.14092945557759</v>
+        <v>12.14093041482172</v>
       </c>
       <c r="D215" t="n">
-        <v>11.82761544584636</v>
+        <v>11.82761638033583</v>
       </c>
       <c r="E215" t="n">
-        <v>11.84328077283316</v>
+        <v>11.84328170856034</v>
       </c>
       <c r="F215" t="n">
         <v>5446800</v>
@@ -4752,16 +4752,16 @@
         <v>44959</v>
       </c>
       <c r="B217" t="n">
-        <v>12.03910160064697</v>
+        <v>12.03910255432129</v>
       </c>
       <c r="C217" t="n">
-        <v>12.19575859750976</v>
+        <v>12.19575956359362</v>
       </c>
       <c r="D217" t="n">
-        <v>11.85111320441163</v>
+        <v>11.8511141431945</v>
       </c>
       <c r="E217" t="n">
-        <v>12.07043300001953</v>
+        <v>12.07043395617575</v>
       </c>
       <c r="F217" t="n">
         <v>3404900</v>
@@ -4932,16 +4932,16 @@
         <v>44972</v>
       </c>
       <c r="B226" t="n">
-        <v>11.75712013244629</v>
+        <v>11.75711917877197</v>
       </c>
       <c r="C226" t="n">
-        <v>11.92944247200145</v>
+        <v>11.92944150434928</v>
       </c>
       <c r="D226" t="n">
-        <v>11.63179452295179</v>
+        <v>11.63179357944321</v>
       </c>
       <c r="E226" t="n">
-        <v>11.66312592532541</v>
+        <v>11.6631249792754</v>
       </c>
       <c r="F226" t="n">
         <v>3961900</v>
@@ -4952,16 +4952,16 @@
         <v>44973</v>
       </c>
       <c r="B227" t="n">
-        <v>11.89027786254883</v>
+        <v>11.89027881622314</v>
       </c>
       <c r="C227" t="n">
-        <v>11.97643902568342</v>
+        <v>11.9764399862684</v>
       </c>
       <c r="D227" t="n">
-        <v>11.57696311596945</v>
+        <v>11.57696404451397</v>
       </c>
       <c r="E227" t="n">
-        <v>11.76495226271687</v>
+        <v>11.7649532063393</v>
       </c>
       <c r="F227" t="n">
         <v>4461000</v>
@@ -5052,16 +5052,16 @@
         <v>44984</v>
       </c>
       <c r="B232" t="n">
-        <v>11.64745998382568</v>
+        <v>11.64745903015137</v>
       </c>
       <c r="C232" t="n">
-        <v>11.85894751251565</v>
+        <v>11.85894654152509</v>
       </c>
       <c r="D232" t="n">
-        <v>11.56129881306286</v>
+        <v>11.56129786644328</v>
       </c>
       <c r="E232" t="n">
-        <v>11.7336211545885</v>
+        <v>11.73362019385946</v>
       </c>
       <c r="F232" t="n">
         <v>3412900</v>
@@ -5092,16 +5092,16 @@
         <v>44986</v>
       </c>
       <c r="B234" t="n">
-        <v>11.52996730804443</v>
+        <v>11.52996635437012</v>
       </c>
       <c r="C234" t="n">
-        <v>11.6552929178602</v>
+        <v>11.65529195381987</v>
       </c>
       <c r="D234" t="n">
-        <v>11.31847978123065</v>
+        <v>11.31847884504903</v>
       </c>
       <c r="E234" t="n">
-        <v>11.6004631503157</v>
+        <v>11.60046219081048</v>
       </c>
       <c r="F234" t="n">
         <v>8005300</v>
@@ -5112,16 +5112,16 @@
         <v>44987</v>
       </c>
       <c r="B235" t="n">
-        <v>11.53779983520508</v>
+        <v>11.53779888153076</v>
       </c>
       <c r="C235" t="n">
-        <v>11.67879152264125</v>
+        <v>11.67879055731306</v>
       </c>
       <c r="D235" t="n">
-        <v>11.45947170096243</v>
+        <v>11.45947075376244</v>
       </c>
       <c r="E235" t="n">
-        <v>11.53779983520508</v>
+        <v>11.53779888153076</v>
       </c>
       <c r="F235" t="n">
         <v>2250800</v>
@@ -5132,16 +5132,16 @@
         <v>44988</v>
       </c>
       <c r="B236" t="n">
-        <v>11.53779983520508</v>
+        <v>11.53779888153076</v>
       </c>
       <c r="C236" t="n">
-        <v>11.64746011954428</v>
+        <v>11.64745915680582</v>
       </c>
       <c r="D236" t="n">
-        <v>11.45947170096243</v>
+        <v>11.45947075376244</v>
       </c>
       <c r="E236" t="n">
-        <v>11.53779983520508</v>
+        <v>11.53779888153076</v>
       </c>
       <c r="F236" t="n">
         <v>1727100</v>
@@ -5172,16 +5172,16 @@
         <v>44992</v>
       </c>
       <c r="B238" t="n">
-        <v>11.61612796783447</v>
+        <v>11.61612701416016</v>
       </c>
       <c r="C238" t="n">
-        <v>11.6239610048538</v>
+        <v>11.6239600505364</v>
       </c>
       <c r="D238" t="n">
-        <v>11.3889751232706</v>
+        <v>11.38897418824534</v>
       </c>
       <c r="E238" t="n">
-        <v>11.52996680162043</v>
+        <v>11.52996585501987</v>
       </c>
       <c r="F238" t="n">
         <v>3776700</v>
@@ -5272,16 +5272,16 @@
         <v>44999</v>
       </c>
       <c r="B243" t="n">
-        <v>11.75712013244629</v>
+        <v>11.75711917877197</v>
       </c>
       <c r="C243" t="n">
-        <v>11.82761597453684</v>
+        <v>11.82761501514428</v>
       </c>
       <c r="D243" t="n">
-        <v>11.63962681329553</v>
+        <v>11.63962586915163</v>
       </c>
       <c r="E243" t="n">
-        <v>11.69445732769904</v>
+        <v>11.69445637910759</v>
       </c>
       <c r="F243" t="n">
         <v>2520000</v>
@@ -5292,16 +5292,16 @@
         <v>45000</v>
       </c>
       <c r="B244" t="n">
-        <v>11.74928569793701</v>
+        <v>11.74928665161133</v>
       </c>
       <c r="C244" t="n">
-        <v>11.89027736535209</v>
+        <v>11.89027833047051</v>
       </c>
       <c r="D244" t="n">
-        <v>11.61612706693377</v>
+        <v>11.61612800979977</v>
       </c>
       <c r="E244" t="n">
-        <v>11.71795429928916</v>
+        <v>11.71795525042035</v>
       </c>
       <c r="F244" t="n">
         <v>4602600</v>
@@ -5372,16 +5372,16 @@
         <v>45006</v>
       </c>
       <c r="B248" t="n">
-        <v>11.34197807312012</v>
+        <v>11.3419771194458</v>
       </c>
       <c r="C248" t="n">
-        <v>11.42030695224922</v>
+        <v>11.42030599198873</v>
       </c>
       <c r="D248" t="n">
-        <v>11.27931526861666</v>
+        <v>11.27931432021125</v>
       </c>
       <c r="E248" t="n">
-        <v>11.36547718505858</v>
+        <v>11.36547622940837</v>
       </c>
       <c r="F248" t="n">
         <v>2410300</v>
@@ -5412,16 +5412,16 @@
         <v>45008</v>
       </c>
       <c r="B250" t="n">
-        <v>11.18532180786133</v>
+        <v>11.18532085418701</v>
       </c>
       <c r="C250" t="n">
-        <v>11.47513748476884</v>
+        <v>11.47513650638449</v>
       </c>
       <c r="D250" t="n">
-        <v>11.05999619049587</v>
+        <v>11.05999524750697</v>
       </c>
       <c r="E250" t="n">
-        <v>11.39680934741524</v>
+        <v>11.39680837570923</v>
       </c>
       <c r="F250" t="n">
         <v>4422500</v>
@@ -5432,16 +5432,16 @@
         <v>45009</v>
       </c>
       <c r="B251" t="n">
-        <v>11.30281352996826</v>
+        <v>11.30281448364258</v>
       </c>
       <c r="C251" t="n">
-        <v>11.39680772964997</v>
+        <v>11.39680869125504</v>
       </c>
       <c r="D251" t="n">
-        <v>11.11482438360535</v>
+        <v>11.11482532141809</v>
       </c>
       <c r="E251" t="n">
-        <v>11.20881933028655</v>
+        <v>11.20882027603011</v>
       </c>
       <c r="F251" t="n">
         <v>3265300</v>
@@ -5452,16 +5452,16 @@
         <v>45012</v>
       </c>
       <c r="B252" t="n">
-        <v>11.28714752197266</v>
+        <v>11.28714847564697</v>
       </c>
       <c r="C252" t="n">
-        <v>11.42030615904377</v>
+        <v>11.42030712396893</v>
       </c>
       <c r="D252" t="n">
-        <v>11.1931533217459</v>
+        <v>11.19315426747845</v>
       </c>
       <c r="E252" t="n">
-        <v>11.39680779573696</v>
+        <v>11.39680875867669</v>
       </c>
       <c r="F252" t="n">
         <v>2288800</v>
@@ -5472,16 +5472,16 @@
         <v>45013</v>
       </c>
       <c r="B253" t="n">
-        <v>11.42030620574951</v>
+        <v>11.4203052520752</v>
       </c>
       <c r="C253" t="n">
-        <v>11.45163760595323</v>
+        <v>11.45163664966253</v>
       </c>
       <c r="D253" t="n">
-        <v>11.25581616793009</v>
+        <v>11.25581522799183</v>
       </c>
       <c r="E253" t="n">
-        <v>11.31064593153673</v>
+        <v>11.3106449870198</v>
       </c>
       <c r="F253" t="n">
         <v>3302900</v>
@@ -5532,16 +5532,16 @@
         <v>45016</v>
       </c>
       <c r="B256" t="n">
-        <v>11.49080181121826</v>
+        <v>11.49080276489258</v>
       </c>
       <c r="C256" t="n">
-        <v>11.61612740950566</v>
+        <v>11.61612837358132</v>
       </c>
       <c r="D256" t="n">
-        <v>11.30281341378716</v>
+        <v>11.30281435185946</v>
       </c>
       <c r="E256" t="n">
-        <v>11.42813901207456</v>
+        <v>11.42813996054821</v>
       </c>
       <c r="F256" t="n">
         <v>5155800</v>
@@ -5552,16 +5552,16 @@
         <v>45019</v>
       </c>
       <c r="B257" t="n">
-        <v>11.34197807312012</v>
+        <v>11.3419771194458</v>
       </c>
       <c r="C257" t="n">
-        <v>11.58479700082069</v>
+        <v>11.58479602672929</v>
       </c>
       <c r="D257" t="n">
-        <v>11.24798386636493</v>
+        <v>11.24798292059398</v>
       </c>
       <c r="E257" t="n">
-        <v>11.58479700082069</v>
+        <v>11.58479602672929</v>
       </c>
       <c r="F257" t="n">
         <v>6471200</v>
@@ -5592,16 +5592,16 @@
         <v>45021</v>
       </c>
       <c r="B259" t="n">
-        <v>11.49080181121826</v>
+        <v>11.49080276489258</v>
       </c>
       <c r="C259" t="n">
-        <v>11.56913068364763</v>
+        <v>11.56913164382282</v>
       </c>
       <c r="D259" t="n">
-        <v>11.27931430385866</v>
+        <v>11.27931523998066</v>
       </c>
       <c r="E259" t="n">
-        <v>11.55346461036196</v>
+        <v>11.55346556923695</v>
       </c>
       <c r="F259" t="n">
         <v>4689800</v>
@@ -5612,16 +5612,16 @@
         <v>45022</v>
       </c>
       <c r="B260" t="n">
-        <v>11.53779983520508</v>
+        <v>11.53779888153076</v>
       </c>
       <c r="C260" t="n">
-        <v>11.66312619459255</v>
+        <v>11.6631252305592</v>
       </c>
       <c r="D260" t="n">
-        <v>11.47513702901113</v>
+        <v>11.4751360805163</v>
       </c>
       <c r="E260" t="n">
-        <v>11.4908031040594</v>
+        <v>11.49080215426967</v>
       </c>
       <c r="F260" t="n">
         <v>4653400</v>
@@ -5772,16 +5772,16 @@
         <v>45035</v>
       </c>
       <c r="B268" t="n">
-        <v>12.03910160064697</v>
+        <v>12.03910255432129</v>
       </c>
       <c r="C268" t="n">
-        <v>12.06259996342652</v>
+        <v>12.06260091896225</v>
       </c>
       <c r="D268" t="n">
-        <v>11.86677853059817</v>
+        <v>11.86677947062196</v>
       </c>
       <c r="E268" t="n">
-        <v>11.96860576530885</v>
+        <v>11.96860671339886</v>
       </c>
       <c r="F268" t="n">
         <v>3098200</v>
@@ -5792,16 +5792,16 @@
         <v>45036</v>
       </c>
       <c r="B269" t="n">
-        <v>12.09393119812012</v>
+        <v>12.09393215179443</v>
       </c>
       <c r="C269" t="n">
-        <v>12.14092867003875</v>
+        <v>12.14092962741908</v>
       </c>
       <c r="D269" t="n">
-        <v>12.00777003776868</v>
+        <v>12.00777098464871</v>
       </c>
       <c r="E269" t="n">
-        <v>12.06259979917419</v>
+        <v>12.06260075037785</v>
       </c>
       <c r="F269" t="n">
         <v>4813100</v>
@@ -5932,16 +5932,16 @@
         <v>45049</v>
       </c>
       <c r="B276" t="n">
-        <v>12.28975296020508</v>
+        <v>12.28975391387939</v>
       </c>
       <c r="C276" t="n">
-        <v>12.48557439565576</v>
+        <v>12.48557536452565</v>
       </c>
       <c r="D276" t="n">
-        <v>12.28192067050667</v>
+        <v>12.2819216235732</v>
       </c>
       <c r="E276" t="n">
-        <v>12.48557439565576</v>
+        <v>12.48557536452565</v>
       </c>
       <c r="F276" t="n">
         <v>6661600</v>
@@ -5992,16 +5992,16 @@
         <v>45054</v>
       </c>
       <c r="B279" t="n">
-        <v>12.11165904998779</v>
+        <v>12.11165809631348</v>
       </c>
       <c r="C279" t="n">
-        <v>12.58781451078781</v>
+        <v>12.58781351962092</v>
       </c>
       <c r="D279" t="n">
-        <v>12.05105773110397</v>
+        <v>12.05105678220141</v>
       </c>
       <c r="E279" t="n">
-        <v>12.54452750060035</v>
+        <v>12.54452651284189</v>
       </c>
       <c r="F279" t="n">
         <v>5826000</v>
@@ -6032,16 +6032,16 @@
         <v>45056</v>
       </c>
       <c r="B281" t="n">
-        <v>11.86925220489502</v>
+        <v>11.86925315856934</v>
       </c>
       <c r="C281" t="n">
-        <v>12.0510569757826</v>
+        <v>12.05105794406462</v>
       </c>
       <c r="D281" t="n">
-        <v>11.69610500062852</v>
+        <v>11.69610594039075</v>
       </c>
       <c r="E281" t="n">
-        <v>12.0164275349293</v>
+        <v>12.0164285004289</v>
       </c>
       <c r="F281" t="n">
         <v>5308900</v>
@@ -6072,16 +6072,16 @@
         <v>45058</v>
       </c>
       <c r="B283" t="n">
-        <v>12.08568668365479</v>
+        <v>12.0856876373291</v>
       </c>
       <c r="C283" t="n">
-        <v>12.25017632493442</v>
+        <v>12.25017729158851</v>
       </c>
       <c r="D283" t="n">
-        <v>11.99911266679329</v>
+        <v>11.9991136136361</v>
       </c>
       <c r="E283" t="n">
-        <v>12.04239967522403</v>
+        <v>12.0424006254826</v>
       </c>
       <c r="F283" t="n">
         <v>3087800</v>
@@ -6112,16 +6112,16 @@
         <v>45062</v>
       </c>
       <c r="B285" t="n">
-        <v>12.12031555175781</v>
+        <v>12.12031650543213</v>
       </c>
       <c r="C285" t="n">
-        <v>12.30212031805942</v>
+        <v>12.30212128603885</v>
       </c>
       <c r="D285" t="n">
-        <v>12.08568611177803</v>
+        <v>12.08568706272756</v>
       </c>
       <c r="E285" t="n">
-        <v>12.18091686531469</v>
+        <v>12.18091782375736</v>
       </c>
       <c r="F285" t="n">
         <v>2907500</v>
@@ -6132,16 +6132,16 @@
         <v>45063</v>
       </c>
       <c r="B286" t="n">
-        <v>11.98179817199707</v>
+        <v>11.98179912567139</v>
       </c>
       <c r="C286" t="n">
-        <v>12.24151939290137</v>
+        <v>12.24152036724783</v>
       </c>
       <c r="D286" t="n">
-        <v>11.94716873091856</v>
+        <v>11.9471696818366</v>
       </c>
       <c r="E286" t="n">
-        <v>12.12897350298847</v>
+        <v>12.128974468377</v>
       </c>
       <c r="F286" t="n">
         <v>4330800</v>
@@ -6152,16 +6152,16 @@
         <v>45064</v>
       </c>
       <c r="B287" t="n">
-        <v>11.98179817199707</v>
+        <v>11.98179912567139</v>
       </c>
       <c r="C287" t="n">
-        <v>12.05971462083146</v>
+        <v>12.05971558070743</v>
       </c>
       <c r="D287" t="n">
-        <v>11.82596527432829</v>
+        <v>11.82596621559931</v>
       </c>
       <c r="E287" t="n">
-        <v>12.01642761307558</v>
+        <v>12.01642856950617</v>
       </c>
       <c r="F287" t="n">
         <v>4680600</v>
@@ -6172,16 +6172,16 @@
         <v>45065</v>
       </c>
       <c r="B288" t="n">
-        <v>12.09434413909912</v>
+        <v>12.09434509277344</v>
       </c>
       <c r="C288" t="n">
-        <v>12.18091732953242</v>
+        <v>12.18091829003328</v>
       </c>
       <c r="D288" t="n">
-        <v>11.93851124043578</v>
+        <v>11.93851218182222</v>
       </c>
       <c r="E288" t="n">
-        <v>11.99911255630219</v>
+        <v>11.99911350246722</v>
       </c>
       <c r="F288" t="n">
         <v>2962700</v>
@@ -6292,16 +6292,16 @@
         <v>45075</v>
       </c>
       <c r="B294" t="n">
-        <v>12.28480625152588</v>
+        <v>12.28480529785156</v>
       </c>
       <c r="C294" t="n">
-        <v>12.34540839597375</v>
+        <v>12.34540743759487</v>
       </c>
       <c r="D294" t="n">
-        <v>12.16360361389222</v>
+        <v>12.16360266962691</v>
       </c>
       <c r="E294" t="n">
-        <v>12.16360361389222</v>
+        <v>12.16360266962691</v>
       </c>
       <c r="F294" t="n">
         <v>1431900</v>
@@ -6312,16 +6312,16 @@
         <v>45076</v>
       </c>
       <c r="B295" t="n">
-        <v>12.26749134063721</v>
+        <v>12.26749229431152</v>
       </c>
       <c r="C295" t="n">
-        <v>12.3800372312229</v>
+        <v>12.38003819364653</v>
       </c>
       <c r="D295" t="n">
-        <v>12.25017620717894</v>
+        <v>12.25017715950718</v>
       </c>
       <c r="E295" t="n">
-        <v>12.37137966449377</v>
+        <v>12.37138062624436</v>
       </c>
       <c r="F295" t="n">
         <v>1829100</v>
@@ -6392,16 +6392,16 @@
         <v>45082</v>
       </c>
       <c r="B299" t="n">
-        <v>12.0683708190918</v>
+        <v>12.06837177276611</v>
       </c>
       <c r="C299" t="n">
-        <v>12.19823183651883</v>
+        <v>12.1982328004551</v>
       </c>
       <c r="D299" t="n">
-        <v>11.97314006681674</v>
+        <v>11.97314101296568</v>
       </c>
       <c r="E299" t="n">
-        <v>12.17225996328581</v>
+        <v>12.17226092516972</v>
       </c>
       <c r="F299" t="n">
         <v>3442900</v>
@@ -6472,16 +6472,16 @@
         <v>45089</v>
       </c>
       <c r="B303" t="n">
-        <v>12.45795440673828</v>
+        <v>12.45795345306396</v>
       </c>
       <c r="C303" t="n">
-        <v>12.45795440673828</v>
+        <v>12.45795345306396</v>
       </c>
       <c r="D303" t="n">
-        <v>12.25883448851593</v>
+        <v>12.25883355008453</v>
       </c>
       <c r="E303" t="n">
-        <v>12.3800379528961</v>
+        <v>12.3800370051864</v>
       </c>
       <c r="F303" t="n">
         <v>2572800</v>
@@ -6492,16 +6492,16 @@
         <v>45090</v>
       </c>
       <c r="B304" t="n">
-        <v>12.3107795715332</v>
+        <v>12.31077861785889</v>
       </c>
       <c r="C304" t="n">
-        <v>12.5012411047074</v>
+        <v>12.50124013627868</v>
       </c>
       <c r="D304" t="n">
-        <v>12.29346443635495</v>
+        <v>12.29346348402198</v>
       </c>
       <c r="E304" t="n">
-        <v>12.46661165998199</v>
+        <v>12.46661069423589</v>
       </c>
       <c r="F304" t="n">
         <v>1312000</v>
@@ -6532,16 +6532,16 @@
         <v>45092</v>
       </c>
       <c r="B306" t="n">
-        <v>12.4666109085083</v>
+        <v>12.46661186218262</v>
       </c>
       <c r="C306" t="n">
-        <v>12.49258360971007</v>
+        <v>12.49258456537125</v>
       </c>
       <c r="D306" t="n">
-        <v>12.36272258059435</v>
+        <v>12.36272352632139</v>
       </c>
       <c r="E306" t="n">
-        <v>12.45795416707208</v>
+        <v>12.45795512008417</v>
       </c>
       <c r="F306" t="n">
         <v>1266000</v>
@@ -6572,16 +6572,16 @@
         <v>45096</v>
       </c>
       <c r="B308" t="n">
-        <v>12.61378574371338</v>
+        <v>12.6137866973877</v>
       </c>
       <c r="C308" t="n">
-        <v>12.80424808345158</v>
+        <v>12.80424905152594</v>
       </c>
       <c r="D308" t="n">
-        <v>12.38869478834751</v>
+        <v>12.38869572500366</v>
       </c>
       <c r="E308" t="n">
-        <v>12.80424808345158</v>
+        <v>12.80424905152594</v>
       </c>
       <c r="F308" t="n">
         <v>3301400</v>
@@ -6592,16 +6592,16 @@
         <v>45097</v>
       </c>
       <c r="B309" t="n">
-        <v>12.72633171081543</v>
+        <v>12.72633266448975</v>
       </c>
       <c r="C309" t="n">
-        <v>12.89947891815102</v>
+        <v>12.89947988480048</v>
       </c>
       <c r="D309" t="n">
-        <v>12.64841526110666</v>
+        <v>12.64841620894215</v>
       </c>
       <c r="E309" t="n">
-        <v>12.69170226934831</v>
+        <v>12.6917032204276</v>
       </c>
       <c r="F309" t="n">
         <v>3568000</v>
@@ -6612,16 +6612,16 @@
         <v>45098</v>
       </c>
       <c r="B310" t="n">
-        <v>12.86485004425049</v>
+        <v>12.86484909057617</v>
       </c>
       <c r="C310" t="n">
-        <v>12.90813705440186</v>
+        <v>12.90813609751867</v>
       </c>
       <c r="D310" t="n">
-        <v>12.63975907759925</v>
+        <v>12.63975814061098</v>
       </c>
       <c r="E310" t="n">
-        <v>12.75230414810935</v>
+        <v>12.75230320277808</v>
       </c>
       <c r="F310" t="n">
         <v>5022600</v>
@@ -6672,16 +6672,16 @@
         <v>45103</v>
       </c>
       <c r="B313" t="n">
-        <v>12.71767520904541</v>
+        <v>12.71767425537109</v>
       </c>
       <c r="C313" t="n">
-        <v>13.01202589898095</v>
+        <v>13.01202492323384</v>
       </c>
       <c r="D313" t="n">
-        <v>12.66573145531036</v>
+        <v>12.66573050553121</v>
       </c>
       <c r="E313" t="n">
-        <v>12.94276701024684</v>
+        <v>12.94276603969331</v>
       </c>
       <c r="F313" t="n">
         <v>2677600</v>
@@ -6692,16 +6692,16 @@
         <v>45104</v>
       </c>
       <c r="B314" t="n">
-        <v>12.50123977661133</v>
+        <v>12.50124073028564</v>
       </c>
       <c r="C314" t="n">
-        <v>12.83887744603771</v>
+        <v>12.83887842546918</v>
       </c>
       <c r="D314" t="n">
-        <v>12.3973514534719</v>
+        <v>12.39735239922096</v>
       </c>
       <c r="E314" t="n">
-        <v>12.76961856394476</v>
+        <v>12.76961953809272</v>
       </c>
       <c r="F314" t="n">
         <v>3014700</v>
@@ -6792,16 +6792,16 @@
         <v>45111</v>
       </c>
       <c r="B319" t="n">
-        <v>12.34540843963623</v>
+        <v>12.34540748596191</v>
       </c>
       <c r="C319" t="n">
-        <v>12.40600975866739</v>
+        <v>12.40600880031166</v>
       </c>
       <c r="D319" t="n">
-        <v>12.23286254312761</v>
+        <v>12.23286159814739</v>
       </c>
       <c r="E319" t="n">
-        <v>12.38869544992894</v>
+        <v>12.38869449291073</v>
       </c>
       <c r="F319" t="n">
         <v>2230100</v>
@@ -6812,16 +6812,16 @@
         <v>45112</v>
       </c>
       <c r="B320" t="n">
-        <v>12.44063854217529</v>
+        <v>12.44063949584961</v>
       </c>
       <c r="C320" t="n">
-        <v>12.54452686599102</v>
+        <v>12.54452782762921</v>
       </c>
       <c r="D320" t="n">
-        <v>12.24151946126957</v>
+        <v>12.24152039967981</v>
       </c>
       <c r="E320" t="n">
-        <v>12.30212077708766</v>
+        <v>12.30212172014348</v>
       </c>
       <c r="F320" t="n">
         <v>5051100</v>
@@ -6852,16 +6852,16 @@
         <v>45114</v>
       </c>
       <c r="B322" t="n">
-        <v>12.34540843963623</v>
+        <v>12.34540748596191</v>
       </c>
       <c r="C322" t="n">
-        <v>12.48392621206805</v>
+        <v>12.48392524769333</v>
       </c>
       <c r="D322" t="n">
-        <v>12.25883441905082</v>
+        <v>12.25883347206429</v>
       </c>
       <c r="E322" t="n">
-        <v>12.42332489303689</v>
+        <v>12.42332393334358</v>
       </c>
       <c r="F322" t="n">
         <v>2149700</v>
@@ -6872,16 +6872,16 @@
         <v>45117</v>
       </c>
       <c r="B323" t="n">
-        <v>12.38869571685791</v>
+        <v>12.38869476318359</v>
       </c>
       <c r="C323" t="n">
-        <v>12.45795460456609</v>
+        <v>12.45795364556026</v>
       </c>
       <c r="D323" t="n">
-        <v>12.31077926177845</v>
+        <v>12.31077831410209</v>
       </c>
       <c r="E323" t="n">
-        <v>12.38003814948662</v>
+        <v>12.38003719647876</v>
       </c>
       <c r="F323" t="n">
         <v>1514600</v>
@@ -6892,16 +6892,16 @@
         <v>45118</v>
       </c>
       <c r="B324" t="n">
-        <v>12.34540843963623</v>
+        <v>12.34540748596191</v>
       </c>
       <c r="C324" t="n">
-        <v>12.39735219148264</v>
+        <v>12.3973512337957</v>
       </c>
       <c r="D324" t="n">
-        <v>12.23286254312761</v>
+        <v>12.23286159814739</v>
       </c>
       <c r="E324" t="n">
-        <v>12.38869544992894</v>
+        <v>12.38869449291073</v>
       </c>
       <c r="F324" t="n">
         <v>1919200</v>
@@ -6912,16 +6912,16 @@
         <v>45119</v>
       </c>
       <c r="B325" t="n">
-        <v>12.38869571685791</v>
+        <v>12.38869476318359</v>
       </c>
       <c r="C325" t="n">
-        <v>12.45795460456609</v>
+        <v>12.45795364556026</v>
       </c>
       <c r="D325" t="n">
-        <v>12.28480655966458</v>
+        <v>12.28480561398759</v>
       </c>
       <c r="E325" t="n">
-        <v>12.37138058211533</v>
+        <v>12.37137962977392</v>
       </c>
       <c r="F325" t="n">
         <v>1842800</v>
@@ -6932,16 +6932,16 @@
         <v>45120</v>
       </c>
       <c r="B326" t="n">
-        <v>12.44063854217529</v>
+        <v>12.44063949584961</v>
       </c>
       <c r="C326" t="n">
-        <v>12.51855499144484</v>
+        <v>12.51855595109208</v>
       </c>
       <c r="D326" t="n">
-        <v>12.34540778508529</v>
+        <v>12.34540873145941</v>
       </c>
       <c r="E326" t="n">
-        <v>12.4752679834472</v>
+        <v>12.47526893977614</v>
       </c>
       <c r="F326" t="n">
         <v>1737300</v>
@@ -6952,16 +6952,16 @@
         <v>45121</v>
       </c>
       <c r="B327" t="n">
-        <v>12.38003826141357</v>
+        <v>12.38003730773926</v>
       </c>
       <c r="C327" t="n">
-        <v>12.48392659391508</v>
+        <v>12.48392563223791</v>
       </c>
       <c r="D327" t="n">
-        <v>12.33675124979684</v>
+        <v>12.33675029945707</v>
       </c>
       <c r="E327" t="n">
-        <v>12.48392659391508</v>
+        <v>12.48392563223791</v>
       </c>
       <c r="F327" t="n">
         <v>1319400</v>
@@ -7052,16 +7052,16 @@
         <v>45128</v>
       </c>
       <c r="B332" t="n">
-        <v>12.38869571685791</v>
+        <v>12.38869476318359</v>
       </c>
       <c r="C332" t="n">
-        <v>12.38869571685791</v>
+        <v>12.38869476318359</v>
       </c>
       <c r="D332" t="n">
-        <v>12.2242052393277</v>
+        <v>12.22420429831576</v>
       </c>
       <c r="E332" t="n">
-        <v>12.27614981792436</v>
+        <v>12.27614887291376</v>
       </c>
       <c r="F332" t="n">
         <v>2631400</v>
@@ -7072,16 +7072,16 @@
         <v>45131</v>
       </c>
       <c r="B333" t="n">
-        <v>12.34540843963623</v>
+        <v>12.34540748596191</v>
       </c>
       <c r="C333" t="n">
-        <v>12.42332489303689</v>
+        <v>12.42332393334358</v>
       </c>
       <c r="D333" t="n">
-        <v>12.31943573808198</v>
+        <v>12.31943478641403</v>
       </c>
       <c r="E333" t="n">
-        <v>12.42332489303689</v>
+        <v>12.42332393334358</v>
       </c>
       <c r="F333" t="n">
         <v>1347200</v>
@@ -7132,16 +7132,16 @@
         <v>45134</v>
       </c>
       <c r="B336" t="n">
-        <v>12.08568668365479</v>
+        <v>12.0856876373291</v>
       </c>
       <c r="C336" t="n">
-        <v>12.22420445012837</v>
+        <v>12.22420541473304</v>
       </c>
       <c r="D336" t="n">
-        <v>12.03374210841168</v>
+        <v>12.03374305798708</v>
       </c>
       <c r="E336" t="n">
-        <v>12.18091744169762</v>
+        <v>12.18091840288654</v>
       </c>
       <c r="F336" t="n">
         <v>2852900</v>
@@ -7152,16 +7152,16 @@
         <v>45135</v>
       </c>
       <c r="B337" t="n">
-        <v>12.12031555175781</v>
+        <v>12.12031650543213</v>
       </c>
       <c r="C337" t="n">
-        <v>12.22420387169716</v>
+        <v>12.22420483354582</v>
       </c>
       <c r="D337" t="n">
-        <v>12.05971423820094</v>
+        <v>12.0597151871069</v>
       </c>
       <c r="E337" t="n">
-        <v>12.14628742533491</v>
+        <v>12.14628838105279</v>
       </c>
       <c r="F337" t="n">
         <v>1506100</v>
@@ -7172,16 +7172,16 @@
         <v>45138</v>
       </c>
       <c r="B338" t="n">
-        <v>12.12031555175781</v>
+        <v>12.12031650543213</v>
       </c>
       <c r="C338" t="n">
-        <v>12.20688956452276</v>
+        <v>12.20689052500906</v>
       </c>
       <c r="D338" t="n">
-        <v>12.10300041895243</v>
+        <v>12.10300137126433</v>
       </c>
       <c r="E338" t="n">
-        <v>12.20688956452276</v>
+        <v>12.20689052500906</v>
       </c>
       <c r="F338" t="n">
         <v>1549400</v>
@@ -7192,16 +7192,16 @@
         <v>45139</v>
       </c>
       <c r="B339" t="n">
-        <v>12.12897396087646</v>
+        <v>12.12897491455078</v>
       </c>
       <c r="C339" t="n">
-        <v>12.38003762458143</v>
+        <v>12.38003859799633</v>
       </c>
       <c r="D339" t="n">
-        <v>12.08568695148643</v>
+        <v>12.08568790175718</v>
       </c>
       <c r="E339" t="n">
-        <v>12.12031639387225</v>
+        <v>12.12031734686584</v>
       </c>
       <c r="F339" t="n">
         <v>5884200</v>
@@ -7292,16 +7292,16 @@
         <v>45146</v>
       </c>
       <c r="B344" t="n">
-        <v>12.08568668365479</v>
+        <v>12.0856876373291</v>
       </c>
       <c r="C344" t="n">
-        <v>12.15494556689158</v>
+        <v>12.15494652603107</v>
       </c>
       <c r="D344" t="n">
-        <v>11.92985378355649</v>
+        <v>11.92985472493413</v>
       </c>
       <c r="E344" t="n">
-        <v>11.99045592561195</v>
+        <v>11.99045687177166</v>
       </c>
       <c r="F344" t="n">
         <v>2176400</v>
@@ -7332,16 +7332,16 @@
         <v>45148</v>
       </c>
       <c r="B346" t="n">
-        <v>11.95582675933838</v>
+        <v>11.9558277130127</v>
       </c>
       <c r="C346" t="n">
-        <v>12.09434452900206</v>
+        <v>12.09434549372545</v>
       </c>
       <c r="D346" t="n">
-        <v>11.88656704887551</v>
+        <v>11.88656799702522</v>
       </c>
       <c r="E346" t="n">
-        <v>12.01642807715848</v>
+        <v>12.01642903566675</v>
       </c>
       <c r="F346" t="n">
         <v>2835300</v>
@@ -7452,16 +7452,16 @@
         <v>45156</v>
       </c>
       <c r="B352" t="n">
-        <v>11.77402210235596</v>
+        <v>11.77402114868164</v>
       </c>
       <c r="C352" t="n">
-        <v>11.80865154513102</v>
+        <v>11.80865058865178</v>
       </c>
       <c r="D352" t="n">
-        <v>11.65281863982772</v>
+        <v>11.65281769597066</v>
       </c>
       <c r="E352" t="n">
-        <v>11.71341995827632</v>
+        <v>11.71341900951066</v>
       </c>
       <c r="F352" t="n">
         <v>3061800</v>
@@ -7492,16 +7492,16 @@
         <v>45160</v>
       </c>
       <c r="B354" t="n">
-        <v>11.79999446868896</v>
+        <v>11.79999351501465</v>
       </c>
       <c r="C354" t="n">
-        <v>11.86925335711897</v>
+        <v>11.86925239784715</v>
       </c>
       <c r="D354" t="n">
-        <v>11.73073558025896</v>
+        <v>11.73073463218214</v>
       </c>
       <c r="E354" t="n">
-        <v>11.79133690122745</v>
+        <v>11.79133594825283</v>
       </c>
       <c r="F354" t="n">
         <v>2231700</v>
@@ -7512,16 +7512,16 @@
         <v>45161</v>
       </c>
       <c r="B355" t="n">
-        <v>11.87791061401367</v>
+        <v>11.87790966033936</v>
       </c>
       <c r="C355" t="n">
-        <v>11.89522492285292</v>
+        <v>11.89522396778845</v>
       </c>
       <c r="D355" t="n">
-        <v>11.79133659292425</v>
+        <v>11.79133564620093</v>
       </c>
       <c r="E355" t="n">
-        <v>11.86059547954337</v>
+        <v>11.86059452725928</v>
       </c>
       <c r="F355" t="n">
         <v>2615000</v>
@@ -7532,16 +7532,16 @@
         <v>45162</v>
       </c>
       <c r="B356" t="n">
-        <v>11.97314167022705</v>
+        <v>11.97314071655273</v>
       </c>
       <c r="C356" t="n">
-        <v>11.99911354693815</v>
+        <v>11.99911259119515</v>
       </c>
       <c r="D356" t="n">
-        <v>11.89522521446267</v>
+        <v>11.89522426699448</v>
       </c>
       <c r="E356" t="n">
-        <v>11.90388278191006</v>
+        <v>11.90388183375229</v>
       </c>
       <c r="F356" t="n">
         <v>2322800</v>
@@ -7592,16 +7592,16 @@
         <v>45167</v>
       </c>
       <c r="B359" t="n">
-        <v>12.12031555175781</v>
+        <v>12.12031650543213</v>
       </c>
       <c r="C359" t="n">
-        <v>12.12031555175781</v>
+        <v>12.12031650543213</v>
       </c>
       <c r="D359" t="n">
-        <v>11.97314022543599</v>
+        <v>11.97314116752997</v>
       </c>
       <c r="E359" t="n">
-        <v>11.98179779183868</v>
+        <v>11.98179873461387</v>
       </c>
       <c r="F359" t="n">
         <v>1776800</v>
@@ -7612,16 +7612,16 @@
         <v>45168</v>
       </c>
       <c r="B360" t="n">
-        <v>12.11165904998779</v>
+        <v>12.11165809631348</v>
       </c>
       <c r="C360" t="n">
-        <v>12.19823307036272</v>
+        <v>12.19823210987155</v>
       </c>
       <c r="D360" t="n">
-        <v>12.05971529826767</v>
+        <v>12.05971434868342</v>
       </c>
       <c r="E360" t="n">
-        <v>12.17226119450266</v>
+        <v>12.17226023605652</v>
       </c>
       <c r="F360" t="n">
         <v>1998700</v>
@@ -7632,16 +7632,16 @@
         <v>45169</v>
       </c>
       <c r="B361" t="n">
-        <v>11.78267860412598</v>
+        <v>11.78267955780029</v>
       </c>
       <c r="C361" t="n">
-        <v>12.1203162835374</v>
+        <v>12.12031726453966</v>
       </c>
       <c r="D361" t="n">
-        <v>11.78267860412598</v>
+        <v>11.78267955780029</v>
       </c>
       <c r="E361" t="n">
-        <v>12.1203162835374</v>
+        <v>12.12031726453966</v>
       </c>
       <c r="F361" t="n">
         <v>3236500</v>
@@ -7652,16 +7652,16 @@
         <v>45170</v>
       </c>
       <c r="B362" t="n">
-        <v>12.04239940643311</v>
+        <v>12.04240036010742</v>
       </c>
       <c r="C362" t="n">
-        <v>12.04239940643311</v>
+        <v>12.04240036010742</v>
       </c>
       <c r="D362" t="n">
-        <v>11.89522407643217</v>
+        <v>11.89522501845123</v>
       </c>
       <c r="E362" t="n">
-        <v>11.90388164305129</v>
+        <v>11.90388258575596</v>
       </c>
       <c r="F362" t="n">
         <v>3740800</v>
@@ -7672,16 +7672,16 @@
         <v>45173</v>
       </c>
       <c r="B363" t="n">
-        <v>12.01642799377441</v>
+        <v>12.01642894744873</v>
       </c>
       <c r="C363" t="n">
-        <v>12.05105743595003</v>
+        <v>12.05105839237269</v>
       </c>
       <c r="D363" t="n">
-        <v>11.81730808204133</v>
+        <v>11.81730901991265</v>
       </c>
       <c r="E363" t="n">
-        <v>12.05105743595003</v>
+        <v>12.05105839237269</v>
       </c>
       <c r="F363" t="n">
         <v>2040600</v>
@@ -7712,16 +7712,16 @@
         <v>45175</v>
       </c>
       <c r="B365" t="n">
-        <v>11.95582675933838</v>
+        <v>11.9558277130127</v>
       </c>
       <c r="C365" t="n">
-        <v>12.02508564417022</v>
+        <v>12.02508660336907</v>
       </c>
       <c r="D365" t="n">
-        <v>11.81730816404367</v>
+        <v>11.81730910666884</v>
       </c>
       <c r="E365" t="n">
-        <v>11.9385116253149</v>
+        <v>11.93851257760805</v>
       </c>
       <c r="F365" t="n">
         <v>2473500</v>
@@ -7772,16 +7772,16 @@
         <v>45181</v>
       </c>
       <c r="B368" t="n">
-        <v>12.0683708190918</v>
+        <v>12.06837177276611</v>
       </c>
       <c r="C368" t="n">
-        <v>12.15494483070982</v>
+        <v>12.15494579122544</v>
       </c>
       <c r="D368" t="n">
-        <v>11.98179763310474</v>
+        <v>11.98179857993782</v>
       </c>
       <c r="E368" t="n">
-        <v>12.03374137957078</v>
+        <v>12.03374233050859</v>
       </c>
       <c r="F368" t="n">
         <v>2215400</v>
@@ -7792,16 +7792,16 @@
         <v>45182</v>
       </c>
       <c r="B369" t="n">
-        <v>12.0683708190918</v>
+        <v>12.06837177276611</v>
       </c>
       <c r="C369" t="n">
-        <v>12.19823183651883</v>
+        <v>12.1982328004551</v>
       </c>
       <c r="D369" t="n">
-        <v>12.03374137957078</v>
+        <v>12.03374233050859</v>
       </c>
       <c r="E369" t="n">
-        <v>12.07702838537979</v>
+        <v>12.07702933973825</v>
       </c>
       <c r="F369" t="n">
         <v>1684100</v>
@@ -7812,16 +7812,16 @@
         <v>45183</v>
       </c>
       <c r="B370" t="n">
-        <v>12.21554660797119</v>
+        <v>12.21554756164551</v>
       </c>
       <c r="C370" t="n">
-        <v>12.25017604880902</v>
+        <v>12.25017700518688</v>
       </c>
       <c r="D370" t="n">
-        <v>12.09434397785428</v>
+        <v>12.09434492206624</v>
       </c>
       <c r="E370" t="n">
-        <v>12.09434397785428</v>
+        <v>12.09434492206624</v>
       </c>
       <c r="F370" t="n">
         <v>2498700</v>
@@ -7892,16 +7892,16 @@
         <v>45189</v>
       </c>
       <c r="B374" t="n">
-        <v>12.0683708190918</v>
+        <v>12.06837177276611</v>
       </c>
       <c r="C374" t="n">
-        <v>12.14628726442182</v>
+        <v>12.1462882242533</v>
       </c>
       <c r="D374" t="n">
-        <v>11.97314006681674</v>
+        <v>11.97314101296568</v>
       </c>
       <c r="E374" t="n">
-        <v>12.08568595166779</v>
+        <v>12.08568690671039</v>
       </c>
       <c r="F374" t="n">
         <v>2998000</v>
@@ -7912,16 +7912,16 @@
         <v>45190</v>
       </c>
       <c r="B375" t="n">
-        <v>11.95582675933838</v>
+        <v>11.9558277130127</v>
       </c>
       <c r="C375" t="n">
-        <v>12.03374238555092</v>
+        <v>12.0337433454403</v>
       </c>
       <c r="D375" t="n">
-        <v>11.8779103074948</v>
+        <v>11.877911254954</v>
       </c>
       <c r="E375" t="n">
-        <v>12.02508564417022</v>
+        <v>12.02508660336907</v>
       </c>
       <c r="F375" t="n">
         <v>4405700</v>
@@ -7932,16 +7932,16 @@
         <v>45191</v>
       </c>
       <c r="B376" t="n">
-        <v>11.95582675933838</v>
+        <v>11.9558277130127</v>
       </c>
       <c r="C376" t="n">
-        <v>12.10300127038276</v>
+        <v>12.10300223579667</v>
       </c>
       <c r="D376" t="n">
-        <v>11.92985405830317</v>
+        <v>11.92985500990573</v>
       </c>
       <c r="E376" t="n">
-        <v>12.02508564417022</v>
+        <v>12.02508660336907</v>
       </c>
       <c r="F376" t="n">
         <v>2812600</v>
@@ -7952,16 +7952,16 @@
         <v>45194</v>
       </c>
       <c r="B377" t="n">
-        <v>11.80865097045898</v>
+        <v>11.8086519241333</v>
       </c>
       <c r="C377" t="n">
-        <v>11.97314060922783</v>
+        <v>11.97314157618643</v>
       </c>
       <c r="D377" t="n">
-        <v>11.80865097045898</v>
+        <v>11.8086519241333</v>
       </c>
       <c r="E377" t="n">
-        <v>11.95582630149842</v>
+        <v>11.95582726705872</v>
       </c>
       <c r="F377" t="n">
         <v>3691700</v>
@@ -8012,16 +8012,16 @@
         <v>45197</v>
       </c>
       <c r="B380" t="n">
-        <v>11.78267860412598</v>
+        <v>11.78267955780029</v>
       </c>
       <c r="C380" t="n">
-        <v>11.86059505519254</v>
+        <v>11.86059601517331</v>
       </c>
       <c r="D380" t="n">
-        <v>11.73073485383562</v>
+        <v>11.73073580330568</v>
       </c>
       <c r="E380" t="n">
-        <v>11.85193748826714</v>
+        <v>11.85193844754717</v>
       </c>
       <c r="F380" t="n">
         <v>2404900</v>
@@ -8072,16 +8072,16 @@
         <v>45202</v>
       </c>
       <c r="B383" t="n">
-        <v>11.80865097045898</v>
+        <v>11.8086519241333</v>
       </c>
       <c r="C383" t="n">
-        <v>11.91253929372841</v>
+        <v>11.91254025579282</v>
       </c>
       <c r="D383" t="n">
-        <v>11.75670639600877</v>
+        <v>11.75670734548801</v>
       </c>
       <c r="E383" t="n">
-        <v>11.8605947192782</v>
+        <v>11.86059567714752</v>
       </c>
       <c r="F383" t="n">
         <v>2809600</v>
@@ -8092,16 +8092,16 @@
         <v>45203</v>
       </c>
       <c r="B384" t="n">
-        <v>11.77402210235596</v>
+        <v>11.77402114868164</v>
       </c>
       <c r="C384" t="n">
-        <v>11.86059529647809</v>
+        <v>11.86059433579151</v>
       </c>
       <c r="D384" t="n">
-        <v>11.74804940105138</v>
+        <v>11.7480484494808</v>
       </c>
       <c r="E384" t="n">
-        <v>11.80865154513102</v>
+        <v>11.80865058865178</v>
       </c>
       <c r="F384" t="n">
         <v>4367600</v>
@@ -8172,16 +8172,16 @@
         <v>45209</v>
       </c>
       <c r="B388" t="n">
-        <v>12.08568668365479</v>
+        <v>12.0856876373291</v>
       </c>
       <c r="C388" t="n">
-        <v>12.16360313370393</v>
+        <v>12.16360409352659</v>
       </c>
       <c r="D388" t="n">
-        <v>11.9125394755628</v>
+        <v>11.91254041557417</v>
       </c>
       <c r="E388" t="n">
-        <v>11.92985378355649</v>
+        <v>11.92985472493413</v>
       </c>
       <c r="F388" t="n">
         <v>3643400</v>
@@ -8192,16 +8192,16 @@
         <v>45210</v>
       </c>
       <c r="B389" t="n">
-        <v>12.09434413909912</v>
+        <v>12.09434509277344</v>
       </c>
       <c r="C389" t="n">
-        <v>12.18957489626505</v>
+        <v>12.18957585744859</v>
       </c>
       <c r="D389" t="n">
-        <v>12.00777012303482</v>
+        <v>12.00777106988252</v>
       </c>
       <c r="E389" t="n">
-        <v>12.09434413909912</v>
+        <v>12.09434509277344</v>
       </c>
       <c r="F389" t="n">
         <v>3458500</v>
@@ -8212,16 +8212,16 @@
         <v>45212</v>
       </c>
       <c r="B390" t="n">
-        <v>12.02508640289307</v>
+        <v>12.02508544921875</v>
       </c>
       <c r="C390" t="n">
-        <v>12.19823362589739</v>
+        <v>12.19823265849127</v>
       </c>
       <c r="D390" t="n">
-        <v>12.02508640289307</v>
+        <v>12.02508544921875</v>
       </c>
       <c r="E390" t="n">
-        <v>12.0943452920948</v>
+        <v>12.09434433292776</v>
       </c>
       <c r="F390" t="n">
         <v>4555500</v>
@@ -8232,16 +8232,16 @@
         <v>45215</v>
       </c>
       <c r="B391" t="n">
-        <v>11.98179817199707</v>
+        <v>11.98179912567139</v>
       </c>
       <c r="C391" t="n">
-        <v>12.12031593631109</v>
+        <v>12.12031690101054</v>
       </c>
       <c r="D391" t="n">
-        <v>11.98179817199707</v>
+        <v>11.98179912567139</v>
       </c>
       <c r="E391" t="n">
-        <v>12.05971462083146</v>
+        <v>12.05971558070743</v>
       </c>
       <c r="F391" t="n">
         <v>3983600</v>
@@ -8252,16 +8252,16 @@
         <v>45216</v>
       </c>
       <c r="B392" t="n">
-        <v>11.95582675933838</v>
+        <v>11.9558277130127</v>
       </c>
       <c r="C392" t="n">
-        <v>12.10300127038276</v>
+        <v>12.10300223579667</v>
       </c>
       <c r="D392" t="n">
-        <v>11.88656704887551</v>
+        <v>11.88656799702522</v>
       </c>
       <c r="E392" t="n">
-        <v>11.97314106773082</v>
+        <v>11.97314202278624</v>
       </c>
       <c r="F392" t="n">
         <v>5165000</v>
@@ -8292,16 +8292,16 @@
         <v>45218</v>
       </c>
       <c r="B394" t="n">
-        <v>11.67013359069824</v>
+        <v>11.67013263702393</v>
       </c>
       <c r="C394" t="n">
-        <v>11.75670761521626</v>
+        <v>11.75670665446719</v>
       </c>
       <c r="D394" t="n">
-        <v>11.62684740407032</v>
+        <v>11.62684645393332</v>
       </c>
       <c r="E394" t="n">
-        <v>11.66147684875131</v>
+        <v>11.66147589578441</v>
       </c>
       <c r="F394" t="n">
         <v>3066300</v>
@@ -8332,16 +8332,16 @@
         <v>45222</v>
       </c>
       <c r="B396" t="n">
-        <v>11.72207736968994</v>
+        <v>11.72207832336426</v>
       </c>
       <c r="C396" t="n">
-        <v>11.90388214825212</v>
+        <v>11.90388311671755</v>
       </c>
       <c r="D396" t="n">
-        <v>11.72207736968994</v>
+        <v>11.72207832336426</v>
       </c>
       <c r="E396" t="n">
-        <v>11.77402194597815</v>
+        <v>11.77402290387853</v>
       </c>
       <c r="F396" t="n">
         <v>3068100</v>
@@ -8352,16 +8352,16 @@
         <v>45223</v>
       </c>
       <c r="B397" t="n">
-        <v>11.63550281524658</v>
+        <v>11.6355037689209</v>
       </c>
       <c r="C397" t="n">
-        <v>11.81730758543626</v>
+        <v>11.81730855401174</v>
       </c>
       <c r="D397" t="n">
-        <v>11.54892962626116</v>
+        <v>11.54893057283972</v>
       </c>
       <c r="E397" t="n">
-        <v>11.80865084447942</v>
+        <v>11.80865181234537</v>
       </c>
       <c r="F397" t="n">
         <v>3637500</v>
@@ -8452,16 +8452,16 @@
         <v>45230</v>
       </c>
       <c r="B402" t="n">
-        <v>11.61818981170654</v>
+        <v>11.61818885803223</v>
       </c>
       <c r="C402" t="n">
-        <v>11.66147682387321</v>
+        <v>11.6614758666457</v>
       </c>
       <c r="D402" t="n">
-        <v>11.52295904544475</v>
+        <v>11.52295809958741</v>
       </c>
       <c r="E402" t="n">
-        <v>11.52295904544475</v>
+        <v>11.52295809958741</v>
       </c>
       <c r="F402" t="n">
         <v>3290000</v>
@@ -8512,16 +8512,16 @@
         <v>45236</v>
       </c>
       <c r="B405" t="n">
-        <v>12.02508640289307</v>
+        <v>12.02508544921875</v>
       </c>
       <c r="C405" t="n">
-        <v>12.07703015697882</v>
+        <v>12.077029199185</v>
       </c>
       <c r="D405" t="n">
-        <v>11.81730890965679</v>
+        <v>11.8173079724607</v>
       </c>
       <c r="E405" t="n">
-        <v>11.94716994613335</v>
+        <v>11.94716899863836</v>
       </c>
       <c r="F405" t="n">
         <v>2982900</v>
@@ -8592,16 +8592,16 @@
         <v>45240</v>
       </c>
       <c r="B409" t="n">
-        <v>11.78267860412598</v>
+        <v>11.78267955780029</v>
       </c>
       <c r="C409" t="n">
-        <v>11.86059505519254</v>
+        <v>11.86059601517331</v>
       </c>
       <c r="D409" t="n">
-        <v>11.69610541176504</v>
+        <v>11.69610635843224</v>
       </c>
       <c r="E409" t="n">
-        <v>11.69610541176504</v>
+        <v>11.69610635843224</v>
       </c>
       <c r="F409" t="n">
         <v>3430000</v>
@@ -8692,16 +8692,16 @@
         <v>45250</v>
       </c>
       <c r="B414" t="n">
-        <v>12.08568668365479</v>
+        <v>12.0856876373291</v>
       </c>
       <c r="C414" t="n">
-        <v>12.23286201694073</v>
+        <v>12.23286298222856</v>
       </c>
       <c r="D414" t="n">
-        <v>11.99045592561195</v>
+        <v>11.99045687177166</v>
       </c>
       <c r="E414" t="n">
-        <v>12.20689014213468</v>
+        <v>12.20689110537309</v>
       </c>
       <c r="F414" t="n">
         <v>3248400</v>
@@ -8712,16 +8712,16 @@
         <v>45251</v>
       </c>
       <c r="B415" t="n">
-        <v>11.97314167022705</v>
+        <v>11.97314071655273</v>
       </c>
       <c r="C415" t="n">
-        <v>12.09434513759732</v>
+        <v>12.09434417426901</v>
       </c>
       <c r="D415" t="n">
-        <v>11.91254034935745</v>
+        <v>11.9125394005101</v>
       </c>
       <c r="E415" t="n">
-        <v>12.08568757014993</v>
+        <v>12.0856866075112</v>
       </c>
       <c r="F415" t="n">
         <v>2713400</v>
@@ -8732,16 +8732,16 @@
         <v>45252</v>
       </c>
       <c r="B416" t="n">
-        <v>12.4666109085083</v>
+        <v>12.46661186218262</v>
       </c>
       <c r="C416" t="n">
-        <v>12.94276636400384</v>
+        <v>12.94276735410323</v>
       </c>
       <c r="D416" t="n">
-        <v>12.44063903293757</v>
+        <v>12.44063998462508</v>
       </c>
       <c r="E416" t="n">
-        <v>12.81290616051917</v>
+        <v>12.81290714068447</v>
       </c>
       <c r="F416" t="n">
         <v>20875500</v>
@@ -8752,16 +8752,16 @@
         <v>45253</v>
       </c>
       <c r="B417" t="n">
-        <v>12.561842918396</v>
+        <v>12.56184196472168</v>
       </c>
       <c r="C417" t="n">
-        <v>12.76961958122722</v>
+        <v>12.76961861177884</v>
       </c>
       <c r="D417" t="n">
-        <v>12.46661132870839</v>
+        <v>12.46661038226389</v>
       </c>
       <c r="E417" t="n">
-        <v>12.76961958122722</v>
+        <v>12.76961861177884</v>
       </c>
       <c r="F417" t="n">
         <v>9122900</v>
@@ -8832,16 +8832,16 @@
         <v>45259</v>
       </c>
       <c r="B421" t="n">
-        <v>12.561842918396</v>
+        <v>12.56184196472168</v>
       </c>
       <c r="C421" t="n">
-        <v>12.75230444650908</v>
+        <v>12.75230347837524</v>
       </c>
       <c r="D421" t="n">
-        <v>12.561842918396</v>
+        <v>12.56184196472168</v>
       </c>
       <c r="E421" t="n">
-        <v>12.72633257006295</v>
+        <v>12.72633160390085</v>
       </c>
       <c r="F421" t="n">
         <v>5869600</v>
@@ -8852,16 +8852,16 @@
         <v>45260</v>
       </c>
       <c r="B422" t="n">
-        <v>12.71767520904541</v>
+        <v>12.71767425537109</v>
       </c>
       <c r="C422" t="n">
-        <v>12.71767520904541</v>
+        <v>12.71767425537109</v>
       </c>
       <c r="D422" t="n">
-        <v>12.58781499907671</v>
+        <v>12.58781405514036</v>
       </c>
       <c r="E422" t="n">
-        <v>12.6311020109433</v>
+        <v>12.63110106376094</v>
       </c>
       <c r="F422" t="n">
         <v>4162000</v>
@@ -8872,16 +8872,16 @@
         <v>45261</v>
       </c>
       <c r="B423" t="n">
-        <v>12.86485004425049</v>
+        <v>12.86484909057617</v>
       </c>
       <c r="C423" t="n">
-        <v>12.96873837323515</v>
+        <v>12.96873741185957</v>
       </c>
       <c r="D423" t="n">
-        <v>12.70901796358902</v>
+        <v>12.70901702146657</v>
       </c>
       <c r="E423" t="n">
-        <v>12.72633227227094</v>
+        <v>12.72633132886498</v>
       </c>
       <c r="F423" t="n">
         <v>6458300</v>
@@ -8892,16 +8892,16 @@
         <v>45264</v>
       </c>
       <c r="B424" t="n">
-        <v>12.89947891235352</v>
+        <v>12.89947986602783</v>
       </c>
       <c r="C424" t="n">
-        <v>12.98605292879791</v>
+        <v>12.98605388887275</v>
       </c>
       <c r="D424" t="n">
-        <v>12.86484947090196</v>
+        <v>12.86485042201608</v>
       </c>
       <c r="E424" t="n">
-        <v>12.94276592057571</v>
+        <v>12.94276687745029</v>
       </c>
       <c r="F424" t="n">
         <v>7048400</v>
@@ -8912,16 +8912,16 @@
         <v>45265</v>
       </c>
       <c r="B425" t="n">
-        <v>13.15919971466064</v>
+        <v>13.15920066833496</v>
       </c>
       <c r="C425" t="n">
-        <v>13.20248672149667</v>
+        <v>13.20248767830808</v>
       </c>
       <c r="D425" t="n">
-        <v>12.9254511987557</v>
+        <v>12.92545213548978</v>
       </c>
       <c r="E425" t="n">
-        <v>12.96008063909832</v>
+        <v>12.96008157834207</v>
       </c>
       <c r="F425" t="n">
         <v>6696500</v>
@@ -8972,16 +8972,16 @@
         <v>45268</v>
       </c>
       <c r="B428" t="n">
-        <v>12.92545223236084</v>
+        <v>12.92545127868652</v>
       </c>
       <c r="C428" t="n">
-        <v>13.15920076695787</v>
+        <v>13.15919979603697</v>
       </c>
       <c r="D428" t="n">
-        <v>12.86485008769187</v>
+        <v>12.86484913848894</v>
       </c>
       <c r="E428" t="n">
-        <v>13.15920076695787</v>
+        <v>13.15919979603697</v>
       </c>
       <c r="F428" t="n">
         <v>10990100</v>
@@ -9052,16 +9052,16 @@
         <v>45274</v>
       </c>
       <c r="B432" t="n">
-        <v>12.94470119476318</v>
+        <v>12.94470024108887</v>
       </c>
       <c r="C432" t="n">
-        <v>12.9831984112191</v>
+        <v>12.98319745470858</v>
       </c>
       <c r="D432" t="n">
-        <v>12.71371789602766</v>
+        <v>12.71371695937057</v>
       </c>
       <c r="E432" t="n">
-        <v>12.71371789602766</v>
+        <v>12.71371695937057</v>
       </c>
       <c r="F432" t="n">
         <v>5480800</v>
@@ -9092,16 +9092,16 @@
         <v>45278</v>
       </c>
       <c r="B434" t="n">
-        <v>12.8484582901001</v>
+        <v>12.84845733642578</v>
       </c>
       <c r="C434" t="n">
-        <v>13.08906611637279</v>
+        <v>13.0890651448394</v>
       </c>
       <c r="D434" t="n">
-        <v>12.8484582901001</v>
+        <v>12.84845733642578</v>
       </c>
       <c r="E434" t="n">
-        <v>12.98319808539135</v>
+        <v>12.983197121716</v>
       </c>
       <c r="F434" t="n">
         <v>3314300</v>
@@ -9112,16 +9112,16 @@
         <v>45279</v>
       </c>
       <c r="B435" t="n">
-        <v>12.86770534515381</v>
+        <v>12.86770629882812</v>
       </c>
       <c r="C435" t="n">
-        <v>12.94469976958878</v>
+        <v>12.94470072896945</v>
       </c>
       <c r="D435" t="n">
-        <v>12.79071092071883</v>
+        <v>12.7907118686868</v>
       </c>
       <c r="E435" t="n">
-        <v>12.87732987766966</v>
+        <v>12.87733083205729</v>
       </c>
       <c r="F435" t="n">
         <v>4780200</v>
@@ -9232,16 +9232,16 @@
         <v>45288</v>
       </c>
       <c r="B441" t="n">
-        <v>12.80996131896973</v>
+        <v>12.80996036529541</v>
       </c>
       <c r="C441" t="n">
-        <v>12.88695575141803</v>
+        <v>12.88695479201164</v>
       </c>
       <c r="D441" t="n">
-        <v>12.76183956922803</v>
+        <v>12.76183861913627</v>
       </c>
       <c r="E441" t="n">
-        <v>12.88695575141803</v>
+        <v>12.88695479201164</v>
       </c>
       <c r="F441" t="n">
         <v>3487000</v>
@@ -9332,16 +9332,16 @@
         <v>45299</v>
       </c>
       <c r="B446" t="n">
-        <v>13.01207160949707</v>
+        <v>13.01207065582275</v>
       </c>
       <c r="C446" t="n">
-        <v>13.09868965545936</v>
+        <v>13.09868869543668</v>
       </c>
       <c r="D446" t="n">
-        <v>12.88695543042352</v>
+        <v>12.88695448591916</v>
       </c>
       <c r="E446" t="n">
-        <v>12.9543253276762</v>
+        <v>12.95432437823419</v>
       </c>
       <c r="F446" t="n">
         <v>3738800</v>
@@ -9392,16 +9392,16 @@
         <v>45302</v>
       </c>
       <c r="B449" t="n">
-        <v>12.8484582901001</v>
+        <v>12.84845733642578</v>
       </c>
       <c r="C449" t="n">
-        <v>12.94470086990156</v>
+        <v>12.94469990908366</v>
       </c>
       <c r="D449" t="n">
-        <v>12.74259025911866</v>
+        <v>12.74258931330238</v>
       </c>
       <c r="E449" t="n">
-        <v>12.94470086990156</v>
+        <v>12.94469990908366</v>
       </c>
       <c r="F449" t="n">
         <v>4814200</v>
@@ -9412,16 +9412,16 @@
         <v>45303</v>
       </c>
       <c r="B450" t="n">
-        <v>12.77146339416504</v>
+        <v>12.77146434783936</v>
       </c>
       <c r="C450" t="n">
-        <v>12.88695503642984</v>
+        <v>12.88695599872818</v>
       </c>
       <c r="D450" t="n">
-        <v>12.74258979521435</v>
+        <v>12.74259074673261</v>
       </c>
       <c r="E450" t="n">
-        <v>12.84845782234157</v>
+        <v>12.84845878176524</v>
       </c>
       <c r="F450" t="n">
         <v>4041800</v>
@@ -9432,16 +9432,16 @@
         <v>45306</v>
       </c>
       <c r="B451" t="n">
-        <v>12.80996131896973</v>
+        <v>12.80996036529541</v>
       </c>
       <c r="C451" t="n">
-        <v>12.84845853519388</v>
+        <v>12.84845757865353</v>
       </c>
       <c r="D451" t="n">
-        <v>12.74259050219293</v>
+        <v>12.74258955353423</v>
       </c>
       <c r="E451" t="n">
-        <v>12.77146410274557</v>
+        <v>12.77146315193729</v>
       </c>
       <c r="F451" t="n">
         <v>1955800</v>
@@ -9492,16 +9492,16 @@
         <v>45309</v>
       </c>
       <c r="B454" t="n">
-        <v>12.55972862243652</v>
+        <v>12.55972766876221</v>
       </c>
       <c r="C454" t="n">
-        <v>12.77146376499286</v>
+        <v>12.77146279524125</v>
       </c>
       <c r="D454" t="n">
-        <v>12.51160687396745</v>
+        <v>12.51160592394707</v>
       </c>
       <c r="E454" t="n">
-        <v>12.76183923172984</v>
+        <v>12.76183826270904</v>
       </c>
       <c r="F454" t="n">
         <v>6534900</v>
@@ -9532,16 +9532,16 @@
         <v>45313</v>
       </c>
       <c r="B456" t="n">
-        <v>12.61747455596924</v>
+        <v>12.61747360229492</v>
       </c>
       <c r="C456" t="n">
-        <v>12.65597177291335</v>
+        <v>12.65597081632927</v>
       </c>
       <c r="D456" t="n">
-        <v>12.56935372317364</v>
+        <v>12.56935277313647</v>
       </c>
       <c r="E456" t="n">
-        <v>12.60785094011775</v>
+        <v>12.60784998717082</v>
       </c>
       <c r="F456" t="n">
         <v>4490300</v>
@@ -9572,16 +9572,16 @@
         <v>45315</v>
       </c>
       <c r="B458" t="n">
-        <v>12.79071140289307</v>
+        <v>12.79071235656738</v>
       </c>
       <c r="C458" t="n">
-        <v>12.82920861656179</v>
+        <v>12.82920957310646</v>
       </c>
       <c r="D458" t="n">
-        <v>12.64634708109684</v>
+        <v>12.64634802400737</v>
       </c>
       <c r="E458" t="n">
-        <v>12.65597069612954</v>
+        <v>12.6559716397576</v>
       </c>
       <c r="F458" t="n">
         <v>3333600</v>
@@ -9652,16 +9652,16 @@
         <v>45321</v>
       </c>
       <c r="B462" t="n">
-        <v>12.51160621643066</v>
+        <v>12.51160717010498</v>
       </c>
       <c r="C462" t="n">
-        <v>12.63672238873649</v>
+        <v>12.63672335194755</v>
       </c>
       <c r="D462" t="n">
-        <v>12.51160621643066</v>
+        <v>12.51160717010498</v>
       </c>
       <c r="E462" t="n">
-        <v>12.58860064279641</v>
+        <v>12.58860160233948</v>
       </c>
       <c r="F462" t="n">
         <v>3463200</v>
@@ -9672,16 +9672,16 @@
         <v>45322</v>
       </c>
       <c r="B463" t="n">
-        <v>12.68484497070312</v>
+        <v>12.68484401702881</v>
       </c>
       <c r="C463" t="n">
-        <v>12.79071208447197</v>
+        <v>12.79071112283833</v>
       </c>
       <c r="D463" t="n">
-        <v>12.53085610782262</v>
+        <v>12.53085516572552</v>
       </c>
       <c r="E463" t="n">
-        <v>12.57897693908826</v>
+        <v>12.57897599337333</v>
       </c>
       <c r="F463" t="n">
         <v>3755000</v>
@@ -9812,16 +9812,16 @@
         <v>45331</v>
       </c>
       <c r="B470" t="n">
-        <v>12.48273372650146</v>
+        <v>12.48273468017578</v>
       </c>
       <c r="C470" t="n">
-        <v>12.62709804867886</v>
+        <v>12.62709901338253</v>
       </c>
       <c r="D470" t="n">
-        <v>12.36724208519036</v>
+        <v>12.36724303004117</v>
       </c>
       <c r="E470" t="n">
-        <v>12.36724208519036</v>
+        <v>12.36724303004117</v>
       </c>
       <c r="F470" t="n">
         <v>4943200</v>
@@ -9852,16 +9852,16 @@
         <v>45337</v>
       </c>
       <c r="B472" t="n">
-        <v>12.50198173522949</v>
+        <v>12.50198268890381</v>
       </c>
       <c r="C472" t="n">
-        <v>12.58860069470964</v>
+        <v>12.58860165499141</v>
       </c>
       <c r="D472" t="n">
-        <v>12.41536277574934</v>
+        <v>12.4153637228162</v>
       </c>
       <c r="E472" t="n">
-        <v>12.46348452188787</v>
+        <v>12.46348547262554</v>
       </c>
       <c r="F472" t="n">
         <v>4740900</v>
@@ -9892,16 +9892,16 @@
         <v>45341</v>
       </c>
       <c r="B474" t="n">
-        <v>12.77146339416504</v>
+        <v>12.77146434783936</v>
       </c>
       <c r="C474" t="n">
-        <v>12.85808143747915</v>
+        <v>12.85808239762144</v>
       </c>
       <c r="D474" t="n">
-        <v>12.53085557665187</v>
+        <v>12.53085651235945</v>
       </c>
       <c r="E474" t="n">
-        <v>12.54047919178945</v>
+        <v>12.54048012821565</v>
       </c>
       <c r="F474" t="n">
         <v>4786000</v>
@@ -9972,16 +9972,16 @@
         <v>45345</v>
       </c>
       <c r="B478" t="n">
-        <v>12.41536235809326</v>
+        <v>12.41536331176758</v>
       </c>
       <c r="C478" t="n">
-        <v>12.55010305917923</v>
+        <v>12.55010402320352</v>
       </c>
       <c r="D478" t="n">
-        <v>12.41536235809326</v>
+        <v>12.41536331176758</v>
       </c>
       <c r="E478" t="n">
-        <v>12.52123037960578</v>
+        <v>12.52123134141225</v>
       </c>
       <c r="F478" t="n">
         <v>4574300</v>
@@ -9992,16 +9992,16 @@
         <v>45348</v>
       </c>
       <c r="B479" t="n">
-        <v>12.35761833190918</v>
+        <v>12.35761737823486</v>
       </c>
       <c r="C479" t="n">
-        <v>12.48273451401776</v>
+        <v>12.48273355068785</v>
       </c>
       <c r="D479" t="n">
-        <v>12.33836926488661</v>
+        <v>12.3383683126978</v>
       </c>
       <c r="E479" t="n">
-        <v>12.45386091348391</v>
+        <v>12.45385995238227</v>
       </c>
       <c r="F479" t="n">
         <v>6964500</v>

</xml_diff>